<commit_message>
auto: data update 2026-09-14 17:43 EDT
Score: 64/100
USD/CNY: 6.71
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85347,13 +85347,13 @@
         <v>1.48</v>
       </c>
       <c r="R521" t="n">
-        <v>4.28</v>
+        <v>4.35</v>
       </c>
       <c r="S521" t="n">
-        <v>2.8</v>
+        <v>2.87</v>
       </c>
       <c r="T521" t="n">
-        <v>2.8</v>
+        <v>2.87</v>
       </c>
       <c r="U521" t="n">
         <v>-3.357531583688344</v>
@@ -85365,10 +85365,10 @@
         <v>-1.603017957351371</v>
       </c>
       <c r="X521" t="n">
-        <v>1.128372874073991</v>
+        <v>1.197250761503854</v>
       </c>
       <c r="Y521" t="n">
-        <v>38.95582329317269</v>
+        <v>39.3574297188755</v>
       </c>
       <c r="Z521" t="inlineStr">
         <is>
@@ -85391,7 +85391,7 @@
         <v>1.785714285714286</v>
       </c>
       <c r="AF521" t="n">
-        <v>0.9462528740739939</v>
+        <v>1.015130761503857</v>
       </c>
       <c r="AG521" t="n">
         <v>6.931259412128282</v>
@@ -85464,25 +85464,25 @@
         </is>
       </c>
       <c r="B522" t="n">
-        <v>4.63</v>
+        <v>4.65</v>
       </c>
       <c r="C522" t="n">
         <v>1.2436</v>
       </c>
       <c r="D522" t="n">
-        <v>3.3834</v>
+        <v>3.406400000000001</v>
       </c>
       <c r="E522" t="n">
-        <v>6.706099987030029</v>
+        <v>6.708000183105469</v>
       </c>
       <c r="F522" t="n">
-        <v>6.709149837493896</v>
+        <v>6.706120014190674</v>
       </c>
       <c r="G522" t="n">
         <v>6.6977</v>
       </c>
       <c r="H522" t="n">
-        <v>0.003049850463867188</v>
+        <v>-0.001880168914794922</v>
       </c>
       <c r="I522" t="n">
         <v>99.12000274658203</v>
@@ -85491,49 +85491,49 @@
         <v>0</v>
       </c>
       <c r="K522" t="n">
-        <v>3.3834</v>
+        <v>3.406400000000001</v>
       </c>
       <c r="L522" t="n">
-        <v>3.09854</v>
+        <v>3.09969</v>
       </c>
       <c r="M522" t="n">
-        <v>2.99448</v>
+        <v>2.994863333333333</v>
       </c>
       <c r="N522" t="n">
-        <v>2.837971666666667</v>
+        <v>2.838163333333333</v>
       </c>
       <c r="O522" t="n">
-        <v>99.80000000000001</v>
+        <v>100</v>
       </c>
       <c r="P522" t="n">
-        <v>99.9001996007984</v>
+        <v>100</v>
       </c>
       <c r="Q522" t="n">
         <v>1.48</v>
       </c>
       <c r="R522" t="n">
-        <v>4.28</v>
+        <v>4.35</v>
       </c>
       <c r="S522" t="n">
-        <v>2.8</v>
+        <v>2.87</v>
       </c>
       <c r="T522" t="n">
-        <v>2.8</v>
+        <v>2.87</v>
       </c>
       <c r="U522" t="n">
-        <v>-3.770936241008185</v>
+        <v>-3.701891751410343</v>
       </c>
       <c r="V522" t="n">
         <v>6.5096</v>
       </c>
       <c r="W522" t="n">
-        <v>-2.930167868210609</v>
+        <v>-2.957665141470223</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.255579052970023</v>
+        <v>-0.2163235751241555</v>
       </c>
       <c r="Y522" t="n">
-        <v>7.630522088353414</v>
+        <v>8.835341365461847</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85556,25 +85556,25 @@
         <v>1.984126984126984</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.4376990529700198</v>
+        <v>-0.3984435751241522</v>
       </c>
       <c r="AG522" t="n">
-        <v>6.95898274179919</v>
+        <v>6.956323088568441</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.2528827547691606</v>
+        <v>-0.2483229054629721</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.567838465599584</v>
+        <v>6.559361964677803</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.1382615214304455</v>
+        <v>0.1486382184276662</v>
       </c>
       <c r="AK522" t="n">
         <v>6.617345065810827</v>
       </c>
       <c r="AL522" t="n">
-        <v>0.08875492121920203</v>
+        <v>0.09065511729464149</v>
       </c>
       <c r="AM522" t="n">
         <v>-0.3685435183382903</v>
@@ -85586,13 +85586,13 @@
         <v>0.8313650598704547</v>
       </c>
       <c r="AP522" t="n">
-        <v>2.341940497809787</v>
+        <v>2.437784108534264</v>
       </c>
       <c r="AQ522" t="n">
-        <v>91.59999999999999</v>
+        <v>92</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.005416740220768371</v>
+        <v>-0.005419845950007125</v>
       </c>
       <c r="AS522" t="n">
         <v>6.7778000831604</v>
@@ -85616,10 +85616,10 @@
         <v>3.125</v>
       </c>
       <c r="AZ522" t="n">
-        <v>63.50375</v>
+        <v>63.69374999999999</v>
       </c>
       <c r="BA522" t="n">
-        <v>63.55028270541696</v>
+        <v>63.58828270541697</v>
       </c>
     </row>
   </sheetData>
@@ -85846,7 +85846,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.63</t>
+          <t>4.65</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -85861,7 +85861,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.38</t>
+          <t>3.41</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -85881,12 +85881,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.28</t>
+          <t>4.35</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -85896,12 +85896,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -85936,7 +85936,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.44</t>
+          <t>-0.40</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -85946,7 +85946,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.14</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -85971,7 +85971,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2.34</t>
+          <t>2.44</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-16 17:10 EDT
Score: 64/100
USD/CNY: 6.71
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85677,13 +85677,13 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>4.37</v>
+        <v>4.39</v>
       </c>
       <c r="S523" t="n">
-        <v>2.89</v>
+        <v>2.91</v>
       </c>
       <c r="T523" t="n">
-        <v>2.89</v>
+        <v>2.91</v>
       </c>
       <c r="U523" t="n">
         <v>-3.69078534719845</v>
@@ -85695,10 +85695,10 @@
         <v>-1.63382096890734</v>
       </c>
       <c r="X523" t="n">
-        <v>1.184781054751416</v>
+        <v>1.204454290557644</v>
       </c>
       <c r="Y523" t="n">
-        <v>38.95582329317269</v>
+        <v>39.75903614457831</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85721,7 +85721,7 @@
         <v>10.31746031746032</v>
       </c>
       <c r="AF523" t="n">
-        <v>0.9949310547514134</v>
+        <v>1.014604290557641</v>
       </c>
       <c r="AG523" t="n">
         <v>6.955785239718927</v>
@@ -85794,25 +85794,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.67</v>
+        <v>4.74</v>
       </c>
       <c r="C524" t="n">
         <v>1.2439</v>
       </c>
       <c r="D524" t="n">
-        <v>3.4261</v>
+        <v>3.4961</v>
       </c>
       <c r="E524" t="n">
-        <v>6.708199977874756</v>
+        <v>6.71120023727417</v>
       </c>
       <c r="F524" t="n">
-        <v>6.71012020111084</v>
+        <v>6.711150169372559</v>
       </c>
       <c r="G524" t="n">
         <v>6.694500000000001</v>
       </c>
       <c r="H524" t="n">
-        <v>0.001920223236083984</v>
+        <v>-5.006790161132812e-05</v>
       </c>
       <c r="I524" t="n">
         <v>99.65000152587891</v>
@@ -85821,49 +85821,49 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>3.4261</v>
+        <v>3.4961</v>
       </c>
       <c r="L524" t="n">
-        <v>3.145855</v>
+        <v>3.149355</v>
       </c>
       <c r="M524" t="n">
-        <v>3.013231666666667</v>
+        <v>3.014398333333333</v>
       </c>
       <c r="N524" t="n">
-        <v>2.853261666666667</v>
+        <v>2.853845</v>
       </c>
       <c r="O524" t="n">
-        <v>99.80000000000001</v>
+        <v>100</v>
       </c>
       <c r="P524" t="n">
-        <v>99.9001996007984</v>
+        <v>100</v>
       </c>
       <c r="Q524" t="n">
         <v>1.48</v>
       </c>
       <c r="R524" t="n">
-        <v>4.37</v>
+        <v>4.39</v>
       </c>
       <c r="S524" t="n">
-        <v>2.89</v>
+        <v>2.91</v>
       </c>
       <c r="T524" t="n">
-        <v>2.89</v>
+        <v>2.91</v>
       </c>
       <c r="U524" t="n">
-        <v>-3.685239417692058</v>
+        <v>-3.500404749871521</v>
       </c>
       <c r="V524" t="n">
         <v>6.5063</v>
       </c>
       <c r="W524" t="n">
-        <v>-3.009748942200141</v>
+        <v>-3.053108684436934</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2512749709742801</v>
+        <v>-0.2771401556836972</v>
       </c>
       <c r="Y524" t="n">
-        <v>8.032128514056225</v>
+        <v>7.228915662650603</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85886,25 +85886,25 @@
         <v>10.51587301587302</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4411249709742826</v>
+        <v>-0.4669901556836997</v>
       </c>
       <c r="AG524" t="n">
-        <v>6.955413207677006</v>
+        <v>6.946119409153104</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.2472132298022505</v>
+        <v>-0.2349191718789339</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.579580030173254</v>
+        <v>6.554531836001155</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.1286199477015018</v>
+        <v>0.1566684012730146</v>
       </c>
       <c r="AK524" t="n">
         <v>6.610494673717893</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.09770530415686274</v>
+        <v>0.1007055635562768</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3578313453157061</v>
@@ -85916,13 +85916,13 @@
         <v>0.8295016854680709</v>
       </c>
       <c r="AP524" t="n">
-        <v>2.196676662060358</v>
+        <v>2.451146565317861</v>
       </c>
       <c r="AQ524" t="n">
-        <v>91.59999999999999</v>
+        <v>92.8</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.00352227905831011</v>
+        <v>-0.003535468258052979</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85946,10 +85946,10 @@
         <v>1.020408163265306</v>
       </c>
       <c r="AZ524" t="n">
-        <v>62.76714285714285</v>
+        <v>63.19714285714286</v>
       </c>
       <c r="BA524" t="n">
-        <v>64.07151014229476</v>
+        <v>64.15751014229475</v>
       </c>
     </row>
   </sheetData>
@@ -86176,7 +86176,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.67</t>
+          <t>4.74</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86191,7 +86191,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -86211,12 +86211,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.37</t>
+          <t>4.39</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>2.91</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86226,12 +86226,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86266,17 +86266,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.44</t>
+          <t>-0.47</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86301,7 +86301,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>2.45</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-21 17:54 EDT
Score: 64/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85355,13 +85355,13 @@
         <v>1.48</v>
       </c>
       <c r="R521" t="n">
-        <v>4.4</v>
+        <v>4.44</v>
       </c>
       <c r="S521" t="n">
-        <v>2.92</v>
+        <v>2.96</v>
       </c>
       <c r="T521" t="n">
-        <v>2.92</v>
+        <v>2.96</v>
       </c>
       <c r="U521" t="n">
         <v>-3.213707527966817</v>
@@ -85373,10 +85373,10 @@
         <v>-1.622086764402386</v>
       </c>
       <c r="X521" t="n">
-        <v>1.226541417963922</v>
+        <v>1.265892583258155</v>
       </c>
       <c r="Y521" t="n">
-        <v>40.56224899598394</v>
+        <v>40.96385542168674</v>
       </c>
       <c r="Z521" t="inlineStr">
         <is>
@@ -85399,7 +85399,7 @@
         <v>13.29365079365079</v>
       </c>
       <c r="AF521" t="n">
-        <v>1.03593141796392</v>
+        <v>1.075282583258153</v>
       </c>
       <c r="AG521" t="n">
         <v>6.922956058876853</v>
@@ -85478,10 +85478,10 @@
         <v>1.2629</v>
       </c>
       <c r="D522" t="n">
-        <v>3.5043</v>
+        <v>3.4971</v>
       </c>
       <c r="E522" t="n">
-        <v>6.707399845123291</v>
+        <v>6.697500228881836</v>
       </c>
       <c r="F522" t="n">
         <v>6.692450046539307</v>
@@ -85490,7 +85490,7 @@
         <v>6.6835</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.01494979858398438</v>
+        <v>-0.005050182342529297</v>
       </c>
       <c r="I522" t="n">
         <v>100.2200012207031</v>
@@ -85499,49 +85499,49 @@
         <v>0</v>
       </c>
       <c r="K522" t="n">
-        <v>3.5043</v>
+        <v>3.4971</v>
       </c>
       <c r="L522" t="n">
-        <v>3.22224</v>
+        <v>3.22188</v>
       </c>
       <c r="M522" t="n">
-        <v>3.046043333333333</v>
+        <v>3.045923333333334</v>
       </c>
       <c r="N522" t="n">
-        <v>2.877595833333333</v>
+        <v>2.877535833333333</v>
       </c>
       <c r="O522" t="n">
-        <v>99.80000000000001</v>
+        <v>99.60000000000001</v>
       </c>
       <c r="P522" t="n">
-        <v>99.9001996007984</v>
+        <v>99.8003992015968</v>
       </c>
       <c r="Q522" t="n">
         <v>1.48</v>
       </c>
       <c r="R522" t="n">
-        <v>4.4</v>
+        <v>4.44</v>
       </c>
       <c r="S522" t="n">
-        <v>2.92</v>
+        <v>2.96</v>
       </c>
       <c r="T522" t="n">
-        <v>2.92</v>
+        <v>2.96</v>
       </c>
       <c r="U522" t="n">
-        <v>-3.228386506343815</v>
+        <v>-3.38096901873113</v>
       </c>
       <c r="V522" t="n">
         <v>6.4894</v>
       </c>
       <c r="W522" t="n">
-        <v>-3.250139400617236</v>
+        <v>-3.107132837180637</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.4731455342443791</v>
+        <v>-0.2850895351514504</v>
       </c>
       <c r="Y522" t="n">
-        <v>2.008032128514056</v>
+        <v>6.827309236947791</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85564,25 +85564,25 @@
         <v>13.49206349206349</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.6637555342443813</v>
+        <v>-0.4756995351514526</v>
       </c>
       <c r="AG522" t="n">
         <v>6.923940636649777</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.2165407915264863</v>
+        <v>-0.2264404077679414</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.582503961350143</v>
+        <v>6.584997578269198</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.1248958837731484</v>
+        <v>0.1125026506126376</v>
       </c>
       <c r="AK522" t="n">
         <v>6.597617692444894</v>
       </c>
       <c r="AL522" t="n">
-        <v>0.1097821526783971</v>
+        <v>0.099882536436942</v>
       </c>
       <c r="AM522" t="n">
         <v>-0.3463356832021003</v>
@@ -85594,13 +85594,13 @@
         <v>0.8306795095823858</v>
       </c>
       <c r="AP522" t="n">
-        <v>2.090385314718188</v>
+        <v>1.97993879059241</v>
       </c>
       <c r="AQ522" t="n">
-        <v>93.59999999999999</v>
+        <v>92.8</v>
       </c>
       <c r="AR522" t="n">
-        <v>-0.002581893773049529</v>
+        <v>-0.002524647682665635</v>
       </c>
       <c r="AS522" t="n">
         <v>6.7778000831604</v>
@@ -85624,10 +85624,10 @@
         <v>0.9900990099009901</v>
       </c>
       <c r="AZ522" t="n">
-        <v>63.35653465346535</v>
+        <v>63.04653465346535</v>
       </c>
       <c r="BA522" t="n">
-        <v>63.60330428271104</v>
+        <v>63.54130428271104</v>
       </c>
     </row>
   </sheetData>
@@ -85839,7 +85839,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.71</t>
+          <t>6.70</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -85889,12 +85889,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.40</t>
+          <t>4.44</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.92</t>
+          <t>2.96</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -85904,12 +85904,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.47</t>
+          <t>-0.29</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -85944,22 +85944,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.66</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>0.11</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.11</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -85979,7 +85979,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-21 18:31 EDT
Score: 64/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.697500228881836</v>
       </c>
       <c r="F522" t="n">
-        <v>6.692450046539307</v>
+        <v>6.69212007522583</v>
       </c>
       <c r="G522" t="n">
         <v>6.6835</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.005050182342529297</v>
+        <v>-0.005380153656005859</v>
       </c>
       <c r="I522" t="n">
         <v>100.2200012207031</v>

</xml_diff>

<commit_message>
auto: data update 2026-09-23 14:03 EDT
Score: 83/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85697,16 +85697,16 @@
         <v>-3.579238540153669</v>
       </c>
       <c r="V523" t="n">
-        <v>6.4916</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-3.042434231826618</v>
+        <v>-1.444298250374509</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2088225551428957</v>
+        <v>1.460430477483832</v>
       </c>
       <c r="Y523" t="n">
-        <v>8.835341365461847</v>
+        <v>41.76706827309237</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85717,10 +85717,10 @@
         <v>1.66939</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.63333</v>
+        <v>1.61939</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.38182</v>
+        <v>1.25205</v>
       </c>
       <c r="AD523" t="n">
         <v>0.1883899999999998</v>
@@ -85729,7 +85729,7 @@
         <v>7.142857142857142</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.3972125551428896</v>
+        <v>1.272040477483838</v>
       </c>
       <c r="AG523" t="n">
         <v>6.93494086387199</v>
@@ -85793,6 +85793,171 @@
       </c>
       <c r="BA523" t="n">
         <v>78.91688888888889</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.2682</v>
+      </c>
+      <c r="D524" t="n">
+        <v>3.4444</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.695300102233887</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.7111</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.7011</v>
+      </c>
+      <c r="H524" t="n">
+        <v>0.01579989776611335</v>
+      </c>
+      <c r="I524" t="n">
+        <v>100.4300003051758</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>3.4444</v>
+      </c>
+      <c r="L524" t="n">
+        <v>3.27265</v>
+      </c>
+      <c r="M524" t="n">
+        <v>3.063965</v>
+      </c>
+      <c r="N524" t="n">
+        <v>2.893474166666667</v>
+      </c>
+      <c r="O524" t="n">
+        <v>98.60000000000001</v>
+      </c>
+      <c r="P524" t="n">
+        <v>99.30139720558883</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.4801</v>
+      </c>
+      <c r="R524" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="S524" t="n">
+        <v>2.9699</v>
+      </c>
+      <c r="T524" t="n">
+        <v>2.9699</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-3.624563035912764</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.4991</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-2.930415354622029</v>
+      </c>
+      <c r="X524" t="n">
+        <v>-0.09091883790270927</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>14.05622489959839</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.66939</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.61939</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.25205</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.18929</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>8.333333333333332</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>-0.2802088379026957</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>6.937975474882886</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.242675372648999</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>6.616249366764732</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>0.07905073546915453</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>6.620905916559939</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>0.07439418567394807</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.3408121180913722</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>0.03433821647994224</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.8341069791131722</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>1.649361913860856</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>90.40000000000001</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>-0.003782807896461949</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.6984</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>0.002699999999999925</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>0.002699999999999925</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.01149821826418838</v>
+      </c>
+      <c r="AW524" t="n">
+        <v>-0.01361566074569778</v>
+      </c>
+      <c r="AX524" t="n">
+        <v>0.01315449425591202</v>
+      </c>
+      <c r="AY524" t="n">
+        <v>94.84126984126983</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>94.82444444444444</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>83.33777777777777</v>
       </c>
     </row>
   </sheetData>
@@ -85999,7 +86164,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -86009,14 +86174,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>6.71</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>6.70</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>6.69</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>4.71</t>
@@ -86064,17 +86229,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6.49</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.21</t>
+          <t>-0.09</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>14</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86089,12 +86254,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -86104,12 +86269,12 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.40</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86124,47 +86289,47 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.09</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.343</t>
+          <t>-0.341</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0.0338</t>
+          <t>0.0343</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.832</t>
+          <t>0.834</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.69</t>
+          <t>1.65</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>-0.003</t>
+          <t>-0.004</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.6928</t>
+          <t>6.6984</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>-0.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>-0.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
@@ -86179,7 +86344,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>83</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-09-23 18:08 EDT
Score: 64/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.699600219726562</v>
       </c>
       <c r="F524" t="n">
-        <v>6.709760189056396</v>
+        <v>6.710400104522705</v>
       </c>
       <c r="G524" t="n">
         <v>6.7011</v>
       </c>
       <c r="H524" t="n">
-        <v>0.01015996932983398</v>
+        <v>0.01079988479614258</v>
       </c>
       <c r="I524" t="n">
         <v>100.4300003051758</v>

</xml_diff>

<commit_message>
auto: data update 2026-09-24 17:25 EDT
Score: 65/100
USD/CNY: 6.71
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.4801</v>
       </c>
       <c r="R523" t="n">
-        <v>4.43</v>
+        <v>4.49</v>
       </c>
       <c r="S523" t="n">
-        <v>2.9499</v>
+        <v>3.0099</v>
       </c>
       <c r="T523" t="n">
-        <v>2.9499</v>
+        <v>3.0099</v>
       </c>
       <c r="U523" t="n">
         <v>-3.281686687457288</v>
@@ -85703,10 +85703,10 @@
         <v>-1.507555919966286</v>
       </c>
       <c r="X523" t="n">
-        <v>1.375559352779199</v>
+        <v>1.434654819227221</v>
       </c>
       <c r="Y523" t="n">
-        <v>41.36546184738956</v>
+        <v>41.76706827309237</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>3.968253968253968</v>
       </c>
       <c r="AF523" t="n">
-        <v>1.188079352779203</v>
+        <v>1.247174819227226</v>
       </c>
       <c r="AG523" t="n">
         <v>6.919460108250188</v>
@@ -85802,25 +85802,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.85</v>
+        <v>4.87</v>
       </c>
       <c r="C524" t="n">
         <v>1.2709</v>
       </c>
       <c r="D524" t="n">
-        <v>3.581799999999999</v>
+        <v>3.5991</v>
       </c>
       <c r="E524" t="n">
-        <v>6.699600219726562</v>
+        <v>6.711100101470947</v>
       </c>
       <c r="F524" t="n">
-        <v>6.715240001678467</v>
+        <v>6.713950157165527</v>
       </c>
       <c r="G524" t="n">
         <v>6.704</v>
       </c>
       <c r="H524" t="n">
-        <v>0.0156397819519043</v>
+        <v>0.002850055694580078</v>
       </c>
       <c r="I524" t="n">
         <v>101.0999984741211</v>
@@ -85829,49 +85829,49 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>3.581799999999999</v>
+        <v>3.5991</v>
       </c>
       <c r="L524" t="n">
-        <v>3.31131</v>
+        <v>3.312175</v>
       </c>
       <c r="M524" t="n">
-        <v>3.077736666666667</v>
+        <v>3.078025</v>
       </c>
       <c r="N524" t="n">
-        <v>2.9040225</v>
+        <v>2.904166666666667</v>
       </c>
       <c r="O524" t="n">
-        <v>99.80000000000001</v>
+        <v>100</v>
       </c>
       <c r="P524" t="n">
-        <v>99.9001996007984</v>
+        <v>100</v>
       </c>
       <c r="Q524" t="n">
         <v>1.48</v>
       </c>
       <c r="R524" t="n">
-        <v>4.43</v>
+        <v>4.49</v>
       </c>
       <c r="S524" t="n">
-        <v>2.95</v>
+        <v>3.01</v>
       </c>
       <c r="T524" t="n">
-        <v>2.95</v>
+        <v>3.01</v>
       </c>
       <c r="U524" t="n">
-        <v>-3.227383950263755</v>
+        <v>-3.011195246071284</v>
       </c>
       <c r="V524" t="n">
         <v>6.5014</v>
       </c>
       <c r="W524" t="n">
-        <v>-2.958388757928776</v>
+        <v>-3.124675512215724</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.1394453799050233</v>
+        <v>-0.2549734427142125</v>
       </c>
       <c r="Y524" t="n">
-        <v>11.24497991967871</v>
+        <v>8.032128514056225</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>5.555555555555555</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.3270253799050327</v>
+        <v>-0.4425534427142219</v>
       </c>
       <c r="AG524" t="n">
-        <v>6.915822041949853</v>
+        <v>6.913184428685526</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.2162218222232903</v>
+        <v>-0.2020843272145783</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.596583422649607</v>
+        <v>6.590741224205351</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.1030167970769558</v>
+        <v>0.1203588772655966</v>
       </c>
       <c r="AK524" t="n">
         <v>6.585215519904615</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.1143846998219473</v>
+        <v>0.1258845815663321</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3376993320378761</v>
@@ -85924,13 +85924,13 @@
         <v>0.8346985405592342</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.8429422540836</v>
+        <v>1.994950017607774</v>
       </c>
       <c r="AQ524" t="n">
-        <v>93.8</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="AR524" t="n">
-        <v>-0.001946934137158551</v>
+        <v>-0.002016762708127403</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85954,10 +85954,10 @@
         <v>17.30769230769231</v>
       </c>
       <c r="AZ524" t="n">
-        <v>69.1276923076923</v>
+        <v>69.67769230769231</v>
       </c>
       <c r="BA524" t="n">
-        <v>65.29351776992047</v>
+        <v>65.40351776992047</v>
       </c>
     </row>
   </sheetData>
@@ -86169,22 +86169,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>6.71</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>6.71</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>6.70</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>6.72</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>6.70</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.85</t>
+          <t>4.87</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86199,7 +86199,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.58</t>
+          <t>3.60</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.43</t>
+          <t>4.49</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.95</t>
+          <t>3.01</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.14</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>8</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,22 +86274,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.33</t>
+          <t>-0.44</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.11</t>
+          <t>0.13</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.84</t>
+          <t>1.99</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-09-28 19:47 EDT
Score: 66/100
USD/CNY: 6.71
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.711100101470947</v>
       </c>
       <c r="F522" t="n">
-        <v>6.709849834442139</v>
+        <v>6.709819793701172</v>
       </c>
       <c r="G522" t="n">
         <v>6.699299999999999</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.001250267028808594</v>
+        <v>-0.001280307769775391</v>
       </c>
       <c r="I522" t="n">
         <v>100.9700012207031</v>

</xml_diff>

<commit_message>
auto: data update 2026-09-30 18:08 EDT
Score: 66/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>4.59</v>
+        <v>4.58</v>
       </c>
       <c r="S523" t="n">
-        <v>3.11</v>
+        <v>3.1</v>
       </c>
       <c r="T523" t="n">
-        <v>3.11</v>
+        <v>3.1</v>
       </c>
       <c r="U523" t="n">
         <v>-2.966782550833697</v>
@@ -85703,7 +85703,7 @@
         <v>-1.664604700835715</v>
       </c>
       <c r="X523" t="n">
-        <v>1.368989943395937</v>
+        <v>1.359156403866013</v>
       </c>
       <c r="Y523" t="n">
         <v>42.40000000000001</v>
@@ -85729,7 +85729,7 @@
         <v>5.555555555555555</v>
       </c>
       <c r="AF523" t="n">
-        <v>1.181409943395928</v>
+        <v>1.171576403866004</v>
       </c>
       <c r="AG523" t="n">
         <v>6.909379977300051</v>
@@ -85802,25 +85802,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.89</v>
+        <v>4.88</v>
       </c>
       <c r="C524" t="n">
         <v>1.2665</v>
       </c>
       <c r="D524" t="n">
-        <v>3.631</v>
+        <v>3.6135</v>
       </c>
       <c r="E524" t="n">
-        <v>6.710299968719482</v>
+        <v>6.703000068664551</v>
       </c>
       <c r="F524" t="n">
-        <v>6.709109783172607</v>
+        <v>6.707859992980957</v>
       </c>
       <c r="G524" t="n">
         <v>6.6978</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.001190185546875</v>
+        <v>0.00485992431640625</v>
       </c>
       <c r="I524" t="n">
         <v>101.370002746582</v>
@@ -85829,49 +85829,49 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>3.631</v>
+        <v>3.6135</v>
       </c>
       <c r="L524" t="n">
-        <v>3.41402</v>
+        <v>3.413145</v>
       </c>
       <c r="M524" t="n">
-        <v>3.125241666666667</v>
+        <v>3.12495</v>
       </c>
       <c r="N524" t="n">
-        <v>2.9432225</v>
+        <v>2.943076666666667</v>
       </c>
       <c r="O524" t="n">
-        <v>99.40239043824701</v>
+        <v>99.20318725099601</v>
       </c>
       <c r="P524" t="n">
-        <v>99.70059880239521</v>
+        <v>99.60079840319361</v>
       </c>
       <c r="Q524" t="n">
         <v>1.48</v>
       </c>
       <c r="R524" t="n">
-        <v>4.59</v>
+        <v>4.58</v>
       </c>
       <c r="S524" t="n">
-        <v>3.11</v>
+        <v>3.1</v>
       </c>
       <c r="T524" t="n">
-        <v>3.11</v>
+        <v>3.1</v>
       </c>
       <c r="U524" t="n">
-        <v>-2.603702037084154</v>
+        <v>-2.735030730976538</v>
       </c>
       <c r="V524" t="n">
         <v>6.494</v>
       </c>
       <c r="W524" t="n">
-        <v>-3.223402377356888</v>
+        <v>-3.118007855043781</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2613565464775647</v>
+        <v>-0.1608126148047617</v>
       </c>
       <c r="Y524" t="n">
-        <v>7.2</v>
+        <v>10.4</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>5.753968253968254</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4489365464775741</v>
+        <v>-0.3483926148047711</v>
       </c>
       <c r="AG524" t="n">
-        <v>6.885016185699489</v>
+        <v>6.886329180439905</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.1747162169800065</v>
+        <v>-0.1833291117753539</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.605342050618161</v>
+        <v>6.611019101913204</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.1049579181013209</v>
+        <v>0.09198096675134693</v>
       </c>
       <c r="AK524" t="n">
         <v>6.588937276483217</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.1213626922362652</v>
+        <v>0.1140627921813335</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3244029311452628</v>
@@ -85924,13 +85924,13 @@
         <v>0.8273982911047538</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.78298099230665</v>
+        <v>1.671865830302798</v>
       </c>
       <c r="AQ524" t="n">
-        <v>95.00956175298805</v>
+        <v>94.61115537848605</v>
       </c>
       <c r="AR524" t="n">
-        <v>0.005596248146053244</v>
+        <v>0.005634591405979897</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85954,10 +85954,10 @@
         <v>8.333333333333332</v>
       </c>
       <c r="AZ524" t="n">
-        <v>66.21037184594954</v>
+        <v>66.02112881806109</v>
       </c>
       <c r="BA524" t="n">
-        <v>66.44993479497273</v>
+        <v>66.41208618939503</v>
       </c>
     </row>
   </sheetData>
@@ -86169,14 +86169,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>6.70</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>6.71</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>6.71</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>6.70</t>
@@ -86184,7 +86184,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.89</t>
+          <t>4.88</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86199,7 +86199,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.63</t>
+          <t>3.61</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.59</t>
+          <t>4.58</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>-0.16</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,22 +86274,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.45</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.17</t>
+          <t>-0.18</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.09</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>0.11</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-01 19:02 EDT
Score: 66/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85791,16 +85791,16 @@
         <v>3.6135</v>
       </c>
       <c r="E524" t="n">
-        <v>6.704500198364258</v>
+        <v>6.703000068664551</v>
       </c>
       <c r="F524" t="n">
-        <v>6.714310169219971</v>
+        <v>6.714119911193848</v>
       </c>
       <c r="G524" t="n">
         <v>6.6987</v>
       </c>
       <c r="H524" t="n">
-        <v>0.009809970855712891</v>
+        <v>0.01111984252929688</v>
       </c>
       <c r="I524" t="n">
         <v>101.4499969482422</v>
@@ -85839,19 +85839,19 @@
         <v>3.06</v>
       </c>
       <c r="U524" t="n">
-        <v>-2.825030982725528</v>
+        <v>-2.848043198340978</v>
       </c>
       <c r="V524" t="n">
         <v>6.494</v>
       </c>
       <c r="W524" t="n">
-        <v>-3.139685168711237</v>
+        <v>-3.118007855043781</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2222268753707013</v>
+        <v>-0.1995654116627499</v>
       </c>
       <c r="Y524" t="n">
-        <v>8.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85874,25 +85874,25 @@
         <v>11.9047619047619</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4116168753707017</v>
+        <v>-0.3889554116627503</v>
       </c>
       <c r="AG524" t="n">
         <v>6.893904406204943</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.1894042078406848</v>
+        <v>-0.1909043375403918</v>
       </c>
       <c r="AI524" t="n">
         <v>6.616658914904448</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.08784128345980946</v>
+        <v>0.08634115376010243</v>
       </c>
       <c r="AK524" t="n">
         <v>6.597254850562075</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.1072453478021833</v>
+        <v>0.1057452181024763</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3220352670441077</v>
@@ -85904,13 +85904,13 @@
         <v>0.8256294933527963</v>
       </c>
       <c r="AP524" t="n">
-        <v>1.62167559286609</v>
+        <v>1.608871142950289</v>
       </c>
       <c r="AQ524" t="n">
         <v>94.41195219123506</v>
       </c>
       <c r="AR524" t="n">
-        <v>0.005565815765295573</v>
+        <v>0.005574789909509401</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -86214,7 +86214,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86254,7 +86254,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.41</t>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86289,7 +86289,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>1.61</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-06 15:12 EDT
Score: 82/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85489,10 +85489,10 @@
         <v>-0.0008001983642573762</v>
       </c>
       <c r="I522" t="n">
-        <v>102.1750030517578</v>
+        <v>102.1699981689453</v>
       </c>
       <c r="J522" t="n">
-        <v>0.002403637259378977</v>
+        <v>0.002354536084086867</v>
       </c>
       <c r="K522" t="n">
         <v>3.6135</v>
@@ -85545,22 +85545,22 @@
         </is>
       </c>
       <c r="AA522" t="n">
-        <v>1.70364</v>
+        <v>1.70545</v>
       </c>
       <c r="AB522" t="n">
-        <v>1.63697</v>
+        <v>1.63606</v>
       </c>
       <c r="AC522" t="n">
-        <v>1.24273</v>
+        <v>1.17242</v>
       </c>
       <c r="AD522" t="n">
-        <v>0.2236400000000001</v>
+        <v>0.2254499999999999</v>
       </c>
       <c r="AE522" t="n">
-        <v>29.16666666666666</v>
+        <v>32.14285714285714</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.5233551272357584</v>
+        <v>-0.5251651272357494</v>
       </c>
       <c r="AG522" t="n">
         <v>6.901521507360839</v>
@@ -85569,10 +85569,10 @@
         <v>-0.1970213089965815</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.647248657248133</v>
+        <v>6.647070879651579</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.05725154111612518</v>
+        <v>0.05742931871267842</v>
       </c>
       <c r="AK522" t="n">
         <v>6.604262089192215</v>
@@ -85590,31 +85590,31 @@
         <v>0.8242782676138585</v>
       </c>
       <c r="AP522" t="n">
-        <v>1.342288069789677</v>
+        <v>1.343801616307725</v>
       </c>
       <c r="AQ522" t="n">
         <v>92.61992031872509</v>
       </c>
       <c r="AR522" t="n">
-        <v>0.01044774634271811</v>
+        <v>0.01044395419152776</v>
       </c>
       <c r="AS522" t="n">
-        <v>6.706768420112095</v>
+        <v>6.706764919767332</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.01046842011209481</v>
+        <v>-0.01046491976733233</v>
       </c>
       <c r="AU522" t="n">
         <v>-0.01029999999999998</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.01176925553352031</v>
+        <v>-0.01176908051628218</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.01314260602288992</v>
+        <v>-0.01314254768381054</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.01232577227709983</v>
+        <v>0.01232576352623793</v>
       </c>
       <c r="AY522" t="n">
         <v>62.6984126984127</v>
@@ -85645,16 +85645,16 @@
         <v>6.704500198364258</v>
       </c>
       <c r="F523" t="n">
-        <v>6.7045</v>
+        <v>6.7018</v>
       </c>
       <c r="G523" t="n">
-        <v>6.6963</v>
+        <v>6.6918</v>
       </c>
       <c r="H523" t="n">
-        <v>-1.983642574643341e-07</v>
+        <v>-0.002700198364257389</v>
       </c>
       <c r="I523" t="n">
-        <v>102.1750030517578</v>
+        <v>102.1699981689453</v>
       </c>
       <c r="J523" t="n">
         <v>0</v>
@@ -85710,22 +85710,22 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.70364</v>
+        <v>1.70545</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.63697</v>
+        <v>1.63606</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.24273</v>
+        <v>1.17242</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.2236400000000001</v>
+        <v>0.2254499999999999</v>
       </c>
       <c r="AE523" t="n">
-        <v>29.36507936507936</v>
+        <v>32.34126984126984</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.5233551272357584</v>
+        <v>-0.5251651272357494</v>
       </c>
       <c r="AG523" t="n">
         <v>6.905652796432723</v>
@@ -85734,10 +85734,10 @@
         <v>-0.2011525980684654</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.649723792674285</v>
+        <v>6.649548866368203</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.05477640568997266</v>
+        <v>0.05495133199605462</v>
       </c>
       <c r="AK523" t="n">
         <v>6.607563959811521</v>
@@ -85746,49 +85746,49 @@
         <v>0.09693623855273703</v>
       </c>
       <c r="AM523" t="n">
-        <v>-0.316521011858445</v>
+        <v>-0.3165168044460268</v>
       </c>
       <c r="AN523" t="n">
-        <v>0.03579521415578762</v>
+        <v>0.03579490155954096</v>
       </c>
       <c r="AO523" t="n">
-        <v>0.8235535280548069</v>
+        <v>0.8235490933628323</v>
       </c>
       <c r="AP523" t="n">
-        <v>1.313130887276439</v>
+        <v>1.314599133074133</v>
       </c>
       <c r="AQ523" t="n">
         <v>91.82071713147411</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.01045423381723536</v>
+        <v>0.01045047761259803</v>
       </c>
       <c r="AS523" t="n">
         <v>6.7037</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.007400000000000517</v>
+        <v>-0.01190000000000069</v>
       </c>
       <c r="AU523" t="n">
-        <v>-0.007400000000000517</v>
+        <v>-0.01190000000000069</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.01158629512871334</v>
+        <v>-0.01181112011147523</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01279025894215886</v>
+        <v>-0.01286520060307949</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01221733100034225</v>
+        <v>0.01222856349861843</v>
       </c>
       <c r="AY523" t="n">
-        <v>76.98412698412699</v>
+        <v>55.15873015873017</v>
       </c>
       <c r="AZ523" t="n">
-        <v>88.93289065958388</v>
+        <v>81.29400177069499</v>
       </c>
       <c r="BA523" t="n">
-        <v>83.43037538733952</v>
+        <v>81.90259760956175</v>
       </c>
     </row>
   </sheetData>
@@ -86010,7 +86010,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.70</t>
+          <t>6.69</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -86025,7 +86025,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>102.18</t>
+          <t>102.17</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86080,7 +86080,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -86090,22 +86090,22 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>0.22</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>32</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.52</t>
+          <t>-0.53</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86175,7 +86175,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>82</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-10-06 18:35 EDT
Score: 65/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85516,13 +85516,13 @@
         <v>1.48</v>
       </c>
       <c r="R522" t="n">
-        <v>4.46</v>
+        <v>4.47</v>
       </c>
       <c r="S522" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="T522" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="U522" t="n">
         <v>-2.938642749904761</v>
@@ -85534,10 +85534,10 @@
         <v>-3.139685168711237</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.2997151272357446</v>
+        <v>-0.2900290957526197</v>
       </c>
       <c r="Y522" t="n">
-        <v>7.4</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85560,7 +85560,7 @@
         <v>32.14285714285714</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.5251651272357494</v>
+        <v>-0.5154790957526245</v>
       </c>
       <c r="AG522" t="n">
         <v>6.901521507360839</v>
@@ -85633,7 +85633,7 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>4.84</v>
+        <v>4.79</v>
       </c>
       <c r="C523" t="n">
         <v>1.2665</v>
@@ -85645,13 +85645,13 @@
         <v>6.704500198364258</v>
       </c>
       <c r="F523" t="n">
-        <v>6.701300144195557</v>
+        <v>6.700660228729248</v>
       </c>
       <c r="G523" t="n">
         <v>6.6918</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.003200054168701172</v>
+        <v>-0.003839969635009766</v>
       </c>
       <c r="I523" t="n">
         <v>102.1699981689453</v>
@@ -85681,16 +85681,16 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>4.46</v>
+        <v>4.47</v>
       </c>
       <c r="S523" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="T523" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="U523" t="n">
-        <v>-3.000262392676817</v>
+        <v>-3.098577914587981</v>
       </c>
       <c r="V523" t="n">
         <v>6.494</v>
@@ -85699,10 +85699,10 @@
         <v>-3.139685168711237</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2997151272357446</v>
+        <v>-0.2900290957526197</v>
       </c>
       <c r="Y523" t="n">
-        <v>7.600000000000001</v>
+        <v>7.800000000000001</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85725,13 +85725,13 @@
         <v>32.34126984126984</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.5251651272357494</v>
+        <v>-0.5154790957526245</v>
       </c>
       <c r="AG523" t="n">
-        <v>6.905652796432723</v>
+        <v>6.91224436079428</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.2011525980684654</v>
+        <v>-0.2077441624300223</v>
       </c>
       <c r="AI523" t="n">
         <v>6.649548866368203</v>
@@ -85758,7 +85758,7 @@
         <v>1.314599133074133</v>
       </c>
       <c r="AQ523" t="n">
-        <v>91.82071713147411</v>
+        <v>91.62071713147411</v>
       </c>
       <c r="AR523" t="n">
         <v>0.01045047761259803</v>
@@ -85785,10 +85785,10 @@
         <v>3.571428571428571</v>
       </c>
       <c r="AZ523" t="n">
-        <v>63.23844621513944</v>
+        <v>63.17844621513945</v>
       </c>
       <c r="BA523" t="n">
-        <v>65.27586061401742</v>
+        <v>65.26386061401742</v>
       </c>
     </row>
   </sheetData>
@@ -86015,7 +86015,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.84</t>
+          <t>4.79</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86050,12 +86050,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.46</t>
+          <t>4.47</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86065,7 +86065,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.29</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -86105,12 +86105,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.53</t>
+          <t>-0.52</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.20</t>
+          <t>-0.21</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-08 16:21 EDT
Score: 78/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.48</v>
       </c>
       <c r="R523" t="n">
-        <v>4.46</v>
+        <v>4.42</v>
       </c>
       <c r="S523" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="T523" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="U523" t="n">
         <v>-3.172126619918144</v>
@@ -85703,10 +85703,10 @@
         <v>-1.579539044388345</v>
       </c>
       <c r="X523" t="n">
-        <v>1.330013514231942</v>
+        <v>1.290645329849704</v>
       </c>
       <c r="Y523" t="n">
-        <v>42.8</v>
+        <v>42</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>52.38095238095238</v>
       </c>
       <c r="AF523" t="n">
-        <v>1.075773514231937</v>
+        <v>1.036405329849699</v>
       </c>
       <c r="AG523" t="n">
         <v>6.917175433889035</v>
@@ -85814,13 +85814,13 @@
         <v>6.704500198364258</v>
       </c>
       <c r="F524" t="n">
-        <v>6.704</v>
+        <v>6.7036</v>
       </c>
       <c r="G524" t="n">
         <v>6.6939</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.0005001983642580754</v>
+        <v>-0.0009001983642580313</v>
       </c>
       <c r="I524" t="n">
         <v>102.2399978637695</v>
@@ -85850,13 +85850,13 @@
         <v>1.48</v>
       </c>
       <c r="R524" t="n">
-        <v>4.46</v>
+        <v>4.42</v>
       </c>
       <c r="S524" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="T524" t="n">
-        <v>2.98</v>
+        <v>2.94</v>
       </c>
       <c r="U524" t="n">
         <v>-3.071215415968181</v>
@@ -85868,10 +85868,10 @@
         <v>-3.090464497484979</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2482992140728113</v>
+        <v>-0.2870630282738151</v>
       </c>
       <c r="Y524" t="n">
-        <v>8</v>
+        <v>6.800000000000001</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,7 +85894,7 @@
         <v>52.57936507936508</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.5025392140728169</v>
+        <v>-0.5413030282738207</v>
       </c>
       <c r="AG524" t="n">
         <v>6.910409842020038</v>
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.46</t>
+          <t>4.42</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>2.94</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.29</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.50</t>
+          <t>-0.54</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-12 21:09 EDT
Score: 61/100
USD/CNY: 6.70
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85489,10 +85489,10 @@
         <v>0.07570028305053711</v>
       </c>
       <c r="I522" t="n">
-        <v>102.5439987182617</v>
+        <v>102.5500030517578</v>
       </c>
       <c r="J522" t="n">
-        <v>0.003267778463758919</v>
+        <v>0.003326523533222492</v>
       </c>
       <c r="K522" t="n">
         <v>3.5281</v>
@@ -85569,10 +85569,10 @@
         <v>-0.2133675640916985</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.695677390952069</v>
+        <v>6.695893169159033</v>
       </c>
       <c r="AJ522" t="n">
-        <v>0.006422409157794462</v>
+        <v>0.006206630950829961</v>
       </c>
       <c r="AK522" t="n">
         <v>6.639129347371973</v>
@@ -85590,31 +85590,31 @@
         <v>0.8219592368747402</v>
       </c>
       <c r="AP522" t="n">
-        <v>0.8805143933118951</v>
+        <v>0.8786898708936047</v>
       </c>
       <c r="AQ522" t="n">
         <v>84.84541832669322</v>
       </c>
       <c r="AR522" t="n">
-        <v>0.01111262014482793</v>
+        <v>0.01111659423810708</v>
       </c>
       <c r="AS522" t="n">
-        <v>6.778046209351267</v>
+        <v>6.778050723580009</v>
       </c>
       <c r="AT522" t="n">
-        <v>-0.09594620935126663</v>
+        <v>-0.09595072358000856</v>
       </c>
       <c r="AU522" t="n">
         <v>-0.09570008316040024</v>
       </c>
       <c r="AV522" t="n">
-        <v>-0.08332263381680724</v>
+        <v>-0.08332285952824434</v>
       </c>
       <c r="AW522" t="n">
-        <v>-0.06267600863103674</v>
+        <v>-0.06267608386818244</v>
       </c>
       <c r="AX522" t="n">
-        <v>0.07877630108880596</v>
+        <v>0.07877631237437781</v>
       </c>
       <c r="AY522" t="n">
         <v>0.8620689655172413</v>
@@ -85645,16 +85645,16 @@
         <v>6.702099800109863</v>
       </c>
       <c r="F523" t="n">
-        <v>6.695040225982666</v>
+        <v>6.693079948425293</v>
       </c>
       <c r="G523" t="n">
         <v>6.6831</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.007059574127197266</v>
+        <v>-0.009019851684570312</v>
       </c>
       <c r="I523" t="n">
-        <v>102.5439987182617</v>
+        <v>102.5500030517578</v>
       </c>
       <c r="J523" t="n">
         <v>0</v>
@@ -85734,10 +85734,10 @@
         <v>-0.2138854214649033</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.696029884321234</v>
+        <v>6.696237960153208</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.006069915788629032</v>
+        <v>0.005861839956655679</v>
       </c>
       <c r="AK523" t="n">
         <v>6.64108897361421</v>
@@ -85746,22 +85746,22 @@
         <v>0.06101082649565281</v>
       </c>
       <c r="AM523" t="n">
-        <v>-0.3089521134145395</v>
+        <v>-0.3089533805873333</v>
       </c>
       <c r="AN523" t="n">
-        <v>0.03573344626898267</v>
+        <v>0.03573205115864952</v>
       </c>
       <c r="AO523" t="n">
-        <v>0.8219595625907712</v>
+        <v>0.8219601623924169</v>
       </c>
       <c r="AP523" t="n">
-        <v>0.8745680103970588</v>
+        <v>0.8728235996431588</v>
       </c>
       <c r="AQ523" t="n">
-        <v>84.44621513944223</v>
+        <v>84.24701195219123</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.0111029165237813</v>
+        <v>0.01110689179419444</v>
       </c>
       <c r="AS523" t="n">
         <v>6.7778000831604</v>
@@ -85773,22 +85773,22 @@
         <v>-0.09470008316040079</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.08415496949790606</v>
+        <v>-0.08415519520934316</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.06387579456897073</v>
+        <v>-0.06387586980611643</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.07938427442931253</v>
+        <v>0.07938429700045625</v>
       </c>
       <c r="AY523" t="n">
         <v>2.564102564102564</v>
       </c>
       <c r="AZ523" t="n">
-        <v>59.5579936663602</v>
+        <v>59.49823271018489</v>
       </c>
       <c r="BA523" t="n">
-        <v>60.62419578361501</v>
+        <v>60.61224359237995</v>
       </c>
     </row>
   </sheetData>
@@ -86005,7 +86005,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.70</t>
+          <t>6.69</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -86025,7 +86025,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>102.54</t>
+          <t>102.55</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-13 16:26 EDT
Score: 78/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85351,13 +85351,13 @@
         <v>1.48</v>
       </c>
       <c r="R521" t="n">
-        <v>4.44</v>
+        <v>4.47</v>
       </c>
       <c r="S521" t="n">
-        <v>2.96</v>
+        <v>2.99</v>
       </c>
       <c r="T521" t="n">
-        <v>2.96</v>
+        <v>2.99</v>
       </c>
       <c r="U521" t="n">
         <v>-3.075089946137582</v>
@@ -85369,10 +85369,10 @@
         <v>-1.54428915111301</v>
       </c>
       <c r="X521" t="n">
-        <v>1.347144410577572</v>
+        <v>1.376681123832246</v>
       </c>
       <c r="Y521" t="n">
-        <v>44.8</v>
+        <v>45.2</v>
       </c>
       <c r="Z521" t="inlineStr">
         <is>
@@ -85395,7 +85395,7 @@
         <v>62.6984126984127</v>
       </c>
       <c r="AF521" t="n">
-        <v>1.074414410577562</v>
+        <v>1.103951123832236</v>
       </c>
       <c r="AG521" t="n">
         <v>6.908195397243149</v>
@@ -85516,13 +85516,13 @@
         <v>1.479</v>
       </c>
       <c r="R522" t="n">
-        <v>4.44</v>
+        <v>4.47</v>
       </c>
       <c r="S522" t="n">
-        <v>2.961</v>
+        <v>2.991</v>
       </c>
       <c r="T522" t="n">
-        <v>2.961</v>
+        <v>2.991</v>
       </c>
       <c r="U522" t="n">
         <v>-3.33932239792969</v>
@@ -85534,7 +85534,7 @@
         <v>-1.395695061065727</v>
       </c>
       <c r="X522" t="n">
-        <v>1.50333607822295</v>
+        <v>1.532917369704623</v>
       </c>
       <c r="Y522" t="n">
         <v>47.2</v>
@@ -85560,7 +85560,7 @@
         <v>88.09523809523809</v>
       </c>
       <c r="AF522" t="n">
-        <v>1.207636078222962</v>
+        <v>1.237217369704635</v>
       </c>
       <c r="AG522" t="n">
         <v>6.915467364201562</v>
@@ -85645,13 +85645,13 @@
         <v>6.691999912261963</v>
       </c>
       <c r="F523" t="n">
-        <v>6.6935</v>
+        <v>6.6931</v>
       </c>
       <c r="G523" t="n">
         <v>6.680800000000001</v>
       </c>
       <c r="H523" t="n">
-        <v>0.001500087738037337</v>
+        <v>0.001100087738037381</v>
       </c>
       <c r="I523" t="n">
         <v>102.5800018310547</v>
@@ -85681,13 +85681,13 @@
         <v>1.478</v>
       </c>
       <c r="R523" t="n">
-        <v>4.44</v>
+        <v>4.47</v>
       </c>
       <c r="S523" t="n">
-        <v>2.962000000000001</v>
+        <v>2.992</v>
       </c>
       <c r="T523" t="n">
-        <v>2.962000000000001</v>
+        <v>2.992</v>
       </c>
       <c r="U523" t="n">
         <v>-3.34216212815395</v>
@@ -85699,10 +85699,10 @@
         <v>-3.009562386468834</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.1811869564280588</v>
+        <v>-0.1520898251439862</v>
       </c>
       <c r="Y523" t="n">
-        <v>9.600000000000001</v>
+        <v>10.8</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85725,7 +85725,7 @@
         <v>88.49206349206349</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.477886956428053</v>
+        <v>-0.4487898251439804</v>
       </c>
       <c r="AG523" t="n">
         <v>6.915657398945678</v>
@@ -86050,12 +86050,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.44</t>
+          <t>4.47</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.96</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86065,12 +86065,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.18</t>
+          <t>-0.15</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86105,7 +86105,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.48</t>
+          <t>-0.45</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-13 18:32 EDT
Score: 78/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85633,25 +85633,25 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>4.8</v>
+        <v>4.79</v>
       </c>
       <c r="C523" t="n">
         <v>1.2607</v>
       </c>
       <c r="D523" t="n">
-        <v>3.5281</v>
+        <v>3.5293</v>
       </c>
       <c r="E523" t="n">
         <v>6.691999912261963</v>
       </c>
       <c r="F523" t="n">
-        <v>6.6931</v>
+        <v>6.693</v>
       </c>
       <c r="G523" t="n">
         <v>6.680800000000001</v>
       </c>
       <c r="H523" t="n">
-        <v>0.001100087738037381</v>
+        <v>0.001000087738036726</v>
       </c>
       <c r="I523" t="n">
         <v>102.5800018310547</v>
@@ -85660,22 +85660,22 @@
         <v>0</v>
       </c>
       <c r="K523" t="n">
-        <v>3.5281</v>
+        <v>3.5293</v>
       </c>
       <c r="L523" t="n">
-        <v>3.558055</v>
+        <v>3.558115</v>
       </c>
       <c r="M523" t="n">
-        <v>3.221235</v>
+        <v>3.221255</v>
       </c>
       <c r="N523" t="n">
-        <v>3.022861666666667</v>
+        <v>3.022871666666667</v>
       </c>
       <c r="O523" t="n">
-        <v>95.21912350597609</v>
+        <v>95.61752988047809</v>
       </c>
       <c r="P523" t="n">
-        <v>97.60479041916167</v>
+        <v>97.80439121756487</v>
       </c>
       <c r="Q523" t="n">
         <v>1.478</v>
@@ -85690,7 +85690,7 @@
         <v>2.992</v>
       </c>
       <c r="U523" t="n">
-        <v>-3.34216212815395</v>
+        <v>-3.361886737953616</v>
       </c>
       <c r="V523" t="n">
         <v>6.4906</v>
@@ -85728,16 +85728,16 @@
         <v>-0.4487898251439804</v>
       </c>
       <c r="AG523" t="n">
-        <v>6.915657398945678</v>
+        <v>6.916977369816165</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.2236574866837149</v>
+        <v>-0.2249774575542025</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.696955139961491</v>
+        <v>6.696584337256301</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.004955227699528386</v>
+        <v>-0.004584424994337866</v>
       </c>
       <c r="AK523" t="n">
         <v>6.640885311001325</v>
@@ -85755,7 +85755,7 @@
         <v>0.8221081273705679</v>
       </c>
       <c r="AP523" t="n">
-        <v>0.7820478524317291</v>
+        <v>0.7851833710246712</v>
       </c>
       <c r="AQ523" t="n">
         <v>81.85179282868526</v>
@@ -85785,10 +85785,10 @@
         <v>44.04761904761904</v>
       </c>
       <c r="AZ523" t="n">
-        <v>73.29889774236386</v>
+        <v>73.43833997343958</v>
       </c>
       <c r="BA523" t="n">
-        <v>77.61561133244797</v>
+        <v>77.64349977866313</v>
       </c>
     </row>
   </sheetData>
@@ -86015,7 +86015,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.80</t>
+          <t>4.79</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86035,7 +86035,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>96</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -86140,7 +86140,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.78</t>
+          <t>0.79</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-14 14:13 EDT
Score: 78/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85654,10 +85654,10 @@
         <v>0.001000087738036726</v>
       </c>
       <c r="I523" t="n">
-        <v>102.5800018310547</v>
+        <v>102.1800003051758</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>-0.00389941039909214</v>
       </c>
       <c r="K523" t="n">
         <v>3.5293</v>
@@ -85693,16 +85693,16 @@
         <v>-3.361886737953616</v>
       </c>
       <c r="V523" t="n">
-        <v>6.4906</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-3.009562386468834</v>
+        <v>-1.395695061065727</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.1520898251439862</v>
+        <v>1.533917369704629</v>
       </c>
       <c r="Y523" t="n">
-        <v>10.8</v>
+        <v>47.6</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85710,22 +85710,22 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.7747</v>
+        <v>1.77833</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.7</v>
+        <v>1.68879</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.42318</v>
+        <v>1.43485</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.2967</v>
+        <v>0.30033</v>
       </c>
       <c r="AE523" t="n">
-        <v>88.49206349206349</v>
+        <v>89.68253968253968</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.4487898251439804</v>
+        <v>1.233587369704625</v>
       </c>
       <c r="AG523" t="n">
         <v>6.916977369816165</v>
@@ -85734,10 +85734,10 @@
         <v>-0.2249774575542025</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.696584337256301</v>
+        <v>6.682324387275842</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.004584424994337866</v>
+        <v>0.009675524986120898</v>
       </c>
       <c r="AK523" t="n">
         <v>6.640885311001325</v>
@@ -85755,40 +85755,205 @@
         <v>0.8221081273705679</v>
       </c>
       <c r="AP523" t="n">
-        <v>0.7851833710246712</v>
+        <v>0.9056917058231858</v>
       </c>
       <c r="AQ523" t="n">
-        <v>81.85179282868526</v>
+        <v>84.24223107569722</v>
       </c>
       <c r="AR523" t="n">
-        <v>0.009068562118789987</v>
+        <v>0.008633097115215262</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.6948</v>
+        <v>6.694574626328669</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.01399999999999935</v>
+        <v>-0.01377462632866866</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.01399999999999935</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.0122385005438828</v>
+        <v>-0.01222723186031627</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.01279026164912446</v>
+        <v>-0.01278650542126895</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.01191090278810075</v>
+        <v>0.01191033935392242</v>
       </c>
       <c r="AY523" t="n">
-        <v>44.04761904761904</v>
+        <v>45.23809523809524</v>
       </c>
       <c r="AZ523" t="n">
-        <v>73.43833997343958</v>
+        <v>74.57213811420982</v>
       </c>
       <c r="BA523" t="n">
-        <v>77.64349977866313</v>
+        <v>77.87025940681717</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.2595</v>
+      </c>
+      <c r="D524" t="n">
+        <v>3.5293</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.691999912261963</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.6965</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.686699999999999</v>
+      </c>
+      <c r="H524" t="n">
+        <v>0.00450008773803745</v>
+      </c>
+      <c r="I524" t="n">
+        <v>102.1800003051758</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>3.5293</v>
+      </c>
+      <c r="L524" t="n">
+        <v>3.559775</v>
+      </c>
+      <c r="M524" t="n">
+        <v>3.229325</v>
+      </c>
+      <c r="N524" t="n">
+        <v>3.030086666666667</v>
+      </c>
+      <c r="O524" t="n">
+        <v>95.41832669322709</v>
+      </c>
+      <c r="P524" t="n">
+        <v>97.70459081836327</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.4748</v>
+      </c>
+      <c r="R524" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="S524" t="n">
+        <v>2.9952</v>
+      </c>
+      <c r="T524" t="n">
+        <v>2.9952</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-3.314902800386011</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.4871</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-3.061863642384666</v>
+      </c>
+      <c r="X524" t="n">
+        <v>-0.2035289471992607</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.77833</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.68879</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.43485</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.3035299999999999</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>90.87301587301587</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>-0.5070589471992681</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>6.913833204755364</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.2218332924934012</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>6.682815635623372</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>0.009184276638590561</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>6.642304621559452</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>0.04969529070251077</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.307524083728529</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>0.03543972981745452</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.8222543449765659</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>0.8982523729987828</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>84.44382470119521</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>0.008342092174878095</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.693</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>-0.006300000000000416</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>-0.006300000000000416</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.01166104350429236</v>
+      </c>
+      <c r="AW524" t="n">
+        <v>-0.01275618321128427</v>
+      </c>
+      <c r="AX524" t="n">
+        <v>0.01187310164527699</v>
+      </c>
+      <c r="AY524" t="n">
+        <v>79.36507936507937</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>86.50733953076582</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>77.7645533421868</v>
       </c>
     </row>
   </sheetData>
@@ -85995,7 +86160,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -86005,14 +86170,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>6.70</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>6.69</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>6.68</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>4.79</t>
@@ -86025,7 +86190,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>102.58</t>
+          <t>102.18</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86035,7 +86200,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>95</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -86045,7 +86210,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.48</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -86055,7 +86220,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.99</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86065,12 +86230,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86080,17 +86245,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -86100,12 +86265,12 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>91</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.45</t>
+          <t>-0.51</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86115,7 +86280,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.00</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86125,12 +86290,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.309</t>
+          <t>-0.308</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0.0356</t>
+          <t>0.0354</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -86140,17 +86305,17 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.79</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>0.009</t>
+          <t>0.008</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>6.6948</t>
+          <t>6.6930</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-14 18:08 EDT
Score: 60/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85810,13 +85810,13 @@
         <v>6.691999912261963</v>
       </c>
       <c r="F524" t="n">
-        <v>6.695030212402344</v>
+        <v>6.694220066070557</v>
       </c>
       <c r="G524" t="n">
         <v>6.686699999999999</v>
       </c>
       <c r="H524" t="n">
-        <v>0.003030300140380859</v>
+        <v>0.00222015380859375</v>
       </c>
       <c r="I524" t="n">
         <v>102.1800003051758</v>
@@ -86170,7 +86170,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.70</t>
+          <t>6.69</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-15 14:46 EDT
Score: 75/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85814,13 +85814,13 @@
         <v>6.691999912261963</v>
       </c>
       <c r="F524" t="n">
-        <v>6.6901</v>
+        <v>6.6903</v>
       </c>
       <c r="G524" t="n">
         <v>6.6804</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.001899912261962733</v>
+        <v>-0.001699912261963199</v>
       </c>
       <c r="I524" t="n">
         <v>102.5500030517578</v>

</xml_diff>

<commit_message>
auto: data update 2026-10-15 17:12 EDT
Score: 75/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.4748</v>
       </c>
       <c r="R523" t="n">
-        <v>4.48</v>
+        <v>4.53</v>
       </c>
       <c r="S523" t="n">
-        <v>3.0052</v>
+        <v>3.0552</v>
       </c>
       <c r="T523" t="n">
-        <v>3.0052</v>
+        <v>3.0552</v>
       </c>
       <c r="U523" t="n">
         <v>-3.255772795701707</v>
@@ -85703,7 +85703,7 @@
         <v>-1.395695061065727</v>
       </c>
       <c r="X523" t="n">
-        <v>1.546977800198523</v>
+        <v>1.596279952667978</v>
       </c>
       <c r="Y523" t="n">
         <v>48</v>
@@ -85729,7 +85729,7 @@
         <v>92.06349206349206</v>
       </c>
       <c r="AF523" t="n">
-        <v>1.242537800198518</v>
+        <v>1.291839952667972</v>
       </c>
       <c r="AG523" t="n">
         <v>6.90987622489377</v>
@@ -85811,16 +85811,16 @@
         <v>3.5605</v>
       </c>
       <c r="E524" t="n">
-        <v>6.691999912261963</v>
+        <v>6.692599773406982</v>
       </c>
       <c r="F524" t="n">
-        <v>6.6903</v>
+        <v>6.6895</v>
       </c>
       <c r="G524" t="n">
         <v>6.6804</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.001699912261963199</v>
+        <v>-0.003099773406982642</v>
       </c>
       <c r="I524" t="n">
         <v>102.5500030517578</v>
@@ -85850,28 +85850,28 @@
         <v>1.474</v>
       </c>
       <c r="R524" t="n">
-        <v>4.48</v>
+        <v>4.53</v>
       </c>
       <c r="S524" t="n">
-        <v>3.006</v>
+        <v>3.056</v>
       </c>
       <c r="T524" t="n">
-        <v>3.006</v>
+        <v>3.056</v>
       </c>
       <c r="U524" t="n">
-        <v>-3.157064444207539</v>
+        <v>-3.147818423693921</v>
       </c>
       <c r="V524" t="n">
         <v>6.4877</v>
       </c>
       <c r="W524" t="n">
-        <v>-3.052897712799096</v>
+        <v>-3.061587131224408</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.1836675303324986</v>
+        <v>-0.144277028268891</v>
       </c>
       <c r="Y524" t="n">
-        <v>9.600000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>94.44444444444444</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4889075303325052</v>
+        <v>-0.4495170282688976</v>
       </c>
       <c r="AG524" t="n">
         <v>6.903270662098385</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.2112707498364221</v>
+        <v>-0.2106708886914026</v>
       </c>
       <c r="AI524" t="n">
         <v>6.6867957940142</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.005204118247762679</v>
+        <v>0.00580397939278221</v>
       </c>
       <c r="AK524" t="n">
         <v>6.636571367753017</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.05542854450894552</v>
+        <v>0.05602840565396505</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3061317321911689</v>
@@ -85924,13 +85924,13 @@
         <v>0.8226928127383537</v>
       </c>
       <c r="AP524" t="n">
-        <v>0.8612371351397863</v>
+        <v>0.8662918728776364</v>
       </c>
       <c r="AQ524" t="n">
-        <v>85.44780876494023</v>
+        <v>85.64701195219124</v>
       </c>
       <c r="AR524" t="n">
-        <v>0.008102517913890779</v>
+        <v>0.008097022110291485</v>
       </c>
       <c r="AS524" t="n">
         <v>6.6961</v>
@@ -85954,10 +85954,10 @@
         <v>32.53968253968254</v>
       </c>
       <c r="AZ524" t="n">
-        <v>70.41964586100043</v>
+        <v>70.47940681717573</v>
       </c>
       <c r="BA524" t="n">
-        <v>74.98701460823372</v>
+        <v>74.99896679946877</v>
       </c>
     </row>
   </sheetData>
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.48</t>
+          <t>4.53</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>3.06</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.18</t>
+          <t>-0.14</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.49</t>
+          <t>-0.45</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>0.87</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-16 16:51 EDT
Score: 59/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85685,13 +85685,13 @@
         <v>1.474</v>
       </c>
       <c r="R523" t="n">
-        <v>4.53</v>
+        <v>4.49</v>
       </c>
       <c r="S523" t="n">
-        <v>3.056</v>
+        <v>3.016</v>
       </c>
       <c r="T523" t="n">
-        <v>3.056</v>
+        <v>3.016</v>
       </c>
       <c r="U523" t="n">
         <v>-3.24629358962126</v>
@@ -85703,7 +85703,7 @@
         <v>-1.404533015413378</v>
       </c>
       <c r="X523" t="n">
-        <v>1.587841638988396</v>
+        <v>1.548403452194558</v>
       </c>
       <c r="Y523" t="n">
         <v>48</v>
@@ -85729,7 +85729,7 @@
         <v>95.63492063492063</v>
       </c>
       <c r="AF523" t="n">
-        <v>1.281691638988391</v>
+        <v>1.242253452194553</v>
       </c>
       <c r="AG523" t="n">
         <v>6.9098612108301</v>
@@ -85811,16 +85811,16 @@
         <v>3.512099999999999</v>
       </c>
       <c r="E524" t="n">
-        <v>6.692599773406982</v>
+        <v>6.690899848937988</v>
       </c>
       <c r="F524" t="n">
-        <v>6.686309814453125</v>
+        <v>6.685219764709473</v>
       </c>
       <c r="G524" t="n">
         <v>6.6755</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.006289958953857422</v>
+        <v>-0.005680084228515625</v>
       </c>
       <c r="I524" t="n">
         <v>102</v>
@@ -85850,28 +85850,28 @@
         <v>1.4705</v>
       </c>
       <c r="R524" t="n">
-        <v>4.53</v>
+        <v>4.49</v>
       </c>
       <c r="S524" t="n">
-        <v>3.0595</v>
+        <v>3.0195</v>
       </c>
       <c r="T524" t="n">
-        <v>3.0595</v>
+        <v>3.0195</v>
       </c>
       <c r="U524" t="n">
-        <v>-3.383774572759958</v>
+        <v>-3.410040786880784</v>
       </c>
       <c r="V524" t="n">
         <v>6.4826</v>
       </c>
       <c r="W524" t="n">
-        <v>-3.13779070192447</v>
+        <v>-3.113181390258757</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.2204326207216445</v>
+        <v>-0.2334632346813859</v>
       </c>
       <c r="Y524" t="n">
-        <v>8.800000000000001</v>
+        <v>8</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85894,25 +85894,25 @@
         <v>96.42857142857142</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.5300826207216502</v>
+        <v>-0.5431132346813916</v>
       </c>
       <c r="AG524" t="n">
         <v>6.919062262796118</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.226462489389136</v>
+        <v>-0.2281624138581302</v>
       </c>
       <c r="AI524" t="n">
         <v>6.682808926787405</v>
       </c>
       <c r="AJ524" t="n">
-        <v>0.009790846619577742</v>
+        <v>0.008090922150583602</v>
       </c>
       <c r="AK524" t="n">
         <v>6.649673665797708</v>
       </c>
       <c r="AL524" t="n">
-        <v>0.04292610760927396</v>
+        <v>0.04122618314027982</v>
       </c>
       <c r="AM524" t="n">
         <v>-0.3047953055253113</v>
@@ -85924,13 +85924,13 @@
         <v>0.8233978564140568</v>
       </c>
       <c r="AP524" t="n">
-        <v>0.8952996452762003</v>
+        <v>0.8810020895634111</v>
       </c>
       <c r="AQ524" t="n">
-        <v>83.44302788844621</v>
+        <v>83.04462151394422</v>
       </c>
       <c r="AR524" t="n">
-        <v>0.01018251026454733</v>
+        <v>0.01019385530952889</v>
       </c>
       <c r="AS524" t="n">
         <v>6.7778000831604</v>
@@ -85954,10 +85954,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="AZ524" t="n">
-        <v>58.16322045152722</v>
+        <v>58.04369853917662</v>
       </c>
       <c r="BA524" t="n">
-        <v>58.91465805112599</v>
+        <v>58.89075366865588</v>
       </c>
     </row>
   </sheetData>
@@ -86219,12 +86219,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.53</t>
+          <t>4.49</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.06</t>
+          <t>3.02</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86234,12 +86234,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.23</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86274,7 +86274,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.53</t>
+          <t>-0.54</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86309,7 +86309,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-19 18:50 EDT
Score: 59/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85484,13 +85484,13 @@
         <v>6.690899848937988</v>
       </c>
       <c r="F522" t="n">
-        <v>6.681570053100586</v>
+        <v>6.682050228118896</v>
       </c>
       <c r="G522" t="n">
         <v>6.6695</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.009329795837402344</v>
+        <v>-0.008849620819091797</v>
       </c>
       <c r="I522" t="n">
         <v>101.8399963378906</v>

</xml_diff>

<commit_message>
auto: data update 2026-10-20 17:29 EDT
Score: 58/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85520,13 +85520,13 @@
         <v>1.468</v>
       </c>
       <c r="R522" t="n">
-        <v>4.46</v>
+        <v>4.5</v>
       </c>
       <c r="S522" t="n">
-        <v>2.992</v>
+        <v>3.032</v>
       </c>
       <c r="T522" t="n">
-        <v>2.992</v>
+        <v>3.032</v>
       </c>
       <c r="U522" t="n">
         <v>-3.446962153218775</v>
@@ -85538,7 +85538,7 @@
         <v>-1.379483343374788</v>
       </c>
       <c r="X522" t="n">
-        <v>1.550991699510695</v>
+        <v>1.590439906173335</v>
       </c>
       <c r="Y522" t="n">
         <v>48.8</v>
@@ -85564,7 +85564,7 @@
         <v>96.82539682539682</v>
       </c>
       <c r="AF522" t="n">
-        <v>1.240661699510692</v>
+        <v>1.280109906173332</v>
       </c>
       <c r="AG522" t="n">
         <v>6.921532634440653</v>
@@ -85649,13 +85649,13 @@
         <v>6.690899848937988</v>
       </c>
       <c r="F523" t="n">
-        <v>6.673840045928955</v>
+        <v>6.673850059509277</v>
       </c>
       <c r="G523" t="n">
         <v>6.666399999999999</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.0170598030090332</v>
+        <v>-0.01704978942871094</v>
       </c>
       <c r="I523" t="n">
         <v>101.9800033569336</v>
@@ -85685,13 +85685,13 @@
         <v>1.4618</v>
       </c>
       <c r="R523" t="n">
-        <v>4.46</v>
+        <v>4.5</v>
       </c>
       <c r="S523" t="n">
-        <v>2.9982</v>
+        <v>3.0382</v>
       </c>
       <c r="T523" t="n">
-        <v>2.9982</v>
+        <v>3.0382</v>
       </c>
       <c r="U523" t="n">
         <v>-3.574709899727847</v>
@@ -85703,10 +85703,10 @@
         <v>-3.232746772802475</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.3787272788694729</v>
+        <v>-0.3400203775785871</v>
       </c>
       <c r="Y523" t="n">
-        <v>5.2</v>
+        <v>5.600000000000001</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85729,7 +85729,7 @@
         <v>98.01587301587301</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.6952572788694766</v>
+        <v>-0.6565503775785908</v>
       </c>
       <c r="AG523" t="n">
         <v>6.93008010821885</v>
@@ -86054,12 +86054,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.46</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>3.04</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86069,12 +86069,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.38</t>
+          <t>-0.34</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86109,7 +86109,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.70</t>
+          <t>-0.66</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-20 18:10 EDT
Score: 59/100
USD/CNY: 6.69
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85637,25 +85637,25 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>4.77</v>
+        <v>4.79</v>
       </c>
       <c r="C523" t="n">
         <v>1.243</v>
       </c>
       <c r="D523" t="n">
-        <v>3.517799999999999</v>
+        <v>3.547</v>
       </c>
       <c r="E523" t="n">
         <v>6.690899848937988</v>
       </c>
       <c r="F523" t="n">
-        <v>6.673850059509277</v>
+        <v>6.674059867858887</v>
       </c>
       <c r="G523" t="n">
         <v>6.666399999999999</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.01704978942871094</v>
+        <v>-0.01683998107910156</v>
       </c>
       <c r="I523" t="n">
         <v>101.9800033569336</v>
@@ -85664,22 +85664,22 @@
         <v>0</v>
       </c>
       <c r="K523" t="n">
-        <v>3.517799999999999</v>
+        <v>3.547</v>
       </c>
       <c r="L523" t="n">
-        <v>3.569945</v>
+        <v>3.571405</v>
       </c>
       <c r="M523" t="n">
-        <v>3.2605</v>
+        <v>3.260986666666667</v>
       </c>
       <c r="N523" t="n">
-        <v>3.059795</v>
+        <v>3.060038333333333</v>
       </c>
       <c r="O523" t="n">
-        <v>93.82470119521912</v>
+        <v>95.21912350597609</v>
       </c>
       <c r="P523" t="n">
-        <v>96.9061876247505</v>
+        <v>97.60479041916167</v>
       </c>
       <c r="Q523" t="n">
         <v>1.4618</v>
@@ -85694,7 +85694,7 @@
         <v>3.0382</v>
       </c>
       <c r="U523" t="n">
-        <v>-3.574709899727847</v>
+        <v>-3.535177568065065</v>
       </c>
       <c r="V523" t="n">
         <v>6.4746</v>
@@ -85732,16 +85732,16 @@
         <v>-0.6565503775785908</v>
       </c>
       <c r="AG523" t="n">
-        <v>6.93008010821885</v>
+        <v>6.927435039499343</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.2391802592808618</v>
+        <v>-0.2365351905613551</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.680665320701229</v>
+        <v>6.671858364424218</v>
       </c>
       <c r="AJ523" t="n">
-        <v>0.01023452823675886</v>
+        <v>0.01904148451377008</v>
       </c>
       <c r="AK523" t="n">
         <v>6.650452785050774</v>
@@ -85759,10 +85759,10 @@
         <v>0.8267651411442265</v>
       </c>
       <c r="AP523" t="n">
-        <v>0.8903928012387073</v>
+        <v>0.9642097098574266</v>
       </c>
       <c r="AQ523" t="n">
-        <v>81.64382470119523</v>
+        <v>83.83585657370517</v>
       </c>
       <c r="AR523" t="n">
         <v>0.008252126669699327</v>
@@ -85789,10 +85789,10 @@
         <v>0.819672131147541</v>
       </c>
       <c r="AZ523" t="n">
-        <v>57.6186780745869</v>
+        <v>58.76433544510482</v>
       </c>
       <c r="BA523" t="n">
-        <v>58.39689970355649</v>
+        <v>58.62603117766007</v>
       </c>
     </row>
   </sheetData>
@@ -86019,7 +86019,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.77</t>
+          <t>4.79</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86034,17 +86034,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.52</t>
+          <t>3.55</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>95</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>98</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -86119,7 +86119,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.01</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86144,7 +86144,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.96</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86179,7 +86179,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-10-21 17:30 EDT
Score: 58/100
USD/CNY: 6.68
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -81089,25 +81089,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.79</v>
+        <v>4.81</v>
       </c>
       <c r="C524" t="n">
         <v>1.2497</v>
       </c>
       <c r="D524" t="n">
-        <v>3.547</v>
+        <v>3.5603</v>
       </c>
       <c r="E524" t="n">
-        <v>6.690899848937988</v>
+        <v>6.677899837493896</v>
       </c>
       <c r="F524" t="n">
-        <v>6.675380229949951</v>
+        <v>6.673480033874512</v>
       </c>
       <c r="G524" t="n">
         <v>6.664199999999999</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01551961898803711</v>
+        <v>-0.004419803619384766</v>
       </c>
       <c r="I524" t="n">
         <v>101.7300033569336</v>
@@ -81116,40 +81116,40 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>3.547</v>
+        <v>3.5603</v>
       </c>
       <c r="L524" t="n">
-        <v>3.569665</v>
+        <v>3.57033</v>
       </c>
       <c r="M524" t="n">
-        <v>3.270918333333333</v>
+        <v>3.27114</v>
       </c>
       <c r="N524" t="n">
-        <v>3.068015</v>
+        <v>3.068125833333333</v>
       </c>
       <c r="O524" t="n">
-        <v>95.0199203187251</v>
+        <v>95.21912350597609</v>
       </c>
       <c r="P524" t="n">
-        <v>97.50499001996008</v>
+        <v>97.60479041916167</v>
       </c>
       <c r="Q524" t="n">
         <v>1.451</v>
       </c>
       <c r="R524" t="n">
-        <v>-3.627556524577208</v>
+        <v>-3.789668582422979</v>
       </c>
       <c r="S524" t="n">
         <v>6.4709</v>
       </c>
       <c r="T524" t="n">
-        <v>-3.288045762228942</v>
+        <v>-3.099774517905618</v>
       </c>
       <c r="U524" t="n">
-        <v>-0.1065431542397022</v>
+        <v>0.1101263277831332</v>
       </c>
       <c r="V524" t="n">
-        <v>6</v>
+        <v>15.2</v>
       </c>
       <c r="W524" t="inlineStr">
         <is>
@@ -81172,25 +81172,25 @@
         <v>98.01587301587301</v>
       </c>
       <c r="AC524" t="n">
-        <v>-0.4249331542397039</v>
+        <v>-0.2082636722168685</v>
       </c>
       <c r="AD524" t="n">
-        <v>6.933616022961065</v>
+        <v>6.930970109601078</v>
       </c>
       <c r="AE524" t="n">
-        <v>-0.2427161740230765</v>
+        <v>-0.2530702721071814</v>
       </c>
       <c r="AF524" t="n">
-        <v>6.663786683483156</v>
+        <v>6.659805076787685</v>
       </c>
       <c r="AG524" t="n">
-        <v>0.027113165454832</v>
+        <v>0.01809476070621141</v>
       </c>
       <c r="AH524" t="n">
         <v>6.644866012143364</v>
       </c>
       <c r="AI524" t="n">
-        <v>0.04603383679462425</v>
+        <v>0.03303382535053245</v>
       </c>
       <c r="AJ524" t="n">
         <v>-0.2993689244715327</v>
@@ -81202,13 +81202,13 @@
         <v>0.8279715895827597</v>
       </c>
       <c r="AM524" t="n">
-        <v>1.026498174523019</v>
+        <v>0.9511180252283403</v>
       </c>
       <c r="AN524" t="n">
-        <v>84.63107569721114</v>
+        <v>82.63665338645419</v>
       </c>
       <c r="AO524" t="n">
-        <v>0.007695232294353127</v>
+        <v>0.007754582480401783</v>
       </c>
       <c r="AP524" t="n">
         <v>6.7778000831604</v>
@@ -81232,10 +81232,10 @@
         <v>0.8130081300813009</v>
       </c>
       <c r="AW524" t="n">
-        <v>58.93084766624558</v>
+        <v>58.40224208855633</v>
       </c>
       <c r="AX524" t="n">
-        <v>58.45120807129814</v>
+        <v>58.34548695576029</v>
       </c>
     </row>
   </sheetData>
@@ -81447,12 +81447,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.69</t>
+          <t>6.68</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6.68</t>
+          <t>6.67</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -81462,7 +81462,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.79</t>
+          <t>4.81</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -81477,7 +81477,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.55</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -81512,12 +81512,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.11</t>
+          <t>0.11</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -81552,24 +81552,24 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.42</t>
+          <t>-0.21</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>0.03</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
       <c r="AA2" t="inlineStr">
         <is>
           <t>-0.299</t>
@@ -81587,7 +81587,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-21 18:12 EDT
Score: 58/100
USD/CNY: 6.68
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -81101,13 +81101,13 @@
         <v>6.677899837493896</v>
       </c>
       <c r="F524" t="n">
-        <v>6.673480033874512</v>
+        <v>6.673359870910645</v>
       </c>
       <c r="G524" t="n">
         <v>6.664199999999999</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.004419803619384766</v>
+        <v>-0.004539966583251953</v>
       </c>
       <c r="I524" t="n">
         <v>101.7300033569336</v>

</xml_diff>

<commit_message>
auto: data update 2026-10-22 18:11 EDT
Score: 58/100
USD/CNY: 6.68
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85818,13 +85818,13 @@
         <v>6.677899837493896</v>
       </c>
       <c r="F524" t="n">
-        <v>6.672239780426025</v>
+        <v>6.672450065612793</v>
       </c>
       <c r="G524" t="n">
         <v>6.664</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.005660057067871094</v>
+        <v>-0.005449771881103516</v>
       </c>
       <c r="I524" t="n">
         <v>101.7799987792969</v>

</xml_diff>

<commit_message>
auto: data update 2026-10-23 17:17 EDT
Score: 56/100
USD/CNY: 6.68
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85689,13 +85689,13 @@
         <v>1.4471</v>
       </c>
       <c r="R523" t="n">
-        <v>4.52</v>
+        <v>4.41</v>
       </c>
       <c r="S523" t="n">
-        <v>3.0729</v>
+        <v>2.9629</v>
       </c>
       <c r="T523" t="n">
-        <v>3.0729</v>
+        <v>2.9629</v>
       </c>
       <c r="U523" t="n">
         <v>-4.84359396118304</v>
@@ -85707,10 +85707,10 @@
         <v>-1.187496659483533</v>
       </c>
       <c r="X523" t="n">
-        <v>1.831728491507811</v>
+        <v>1.723034737833262</v>
       </c>
       <c r="Y523" t="n">
-        <v>50.40000000000001</v>
+        <v>50</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85733,7 +85733,7 @@
         <v>98.01587301587301</v>
       </c>
       <c r="AF523" t="n">
-        <v>1.510338491507812</v>
+        <v>1.401644737833263</v>
       </c>
       <c r="AG523" t="n">
         <v>7.001350190756603</v>
@@ -85806,25 +85806,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.65</v>
+        <v>4.69</v>
       </c>
       <c r="C524" t="n">
         <v>1.2452</v>
       </c>
       <c r="D524" t="n">
-        <v>3.404</v>
+        <v>3.4448</v>
       </c>
       <c r="E524" t="n">
         <v>6.677899837493896</v>
       </c>
       <c r="F524" t="n">
-        <v>6.669060230255127</v>
+        <v>6.668200016021729</v>
       </c>
       <c r="G524" t="n">
         <v>6.6596</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.008839607238769531</v>
+        <v>-0.009699821472167969</v>
       </c>
       <c r="I524" t="n">
         <v>101.6100006103516</v>
@@ -85833,37 +85833,37 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>3.404</v>
+        <v>3.4448</v>
       </c>
       <c r="L524" t="n">
-        <v>3.550819999999999</v>
+        <v>3.55286</v>
       </c>
       <c r="M524" t="n">
-        <v>3.284831666666667</v>
+        <v>3.285511666666666</v>
       </c>
       <c r="N524" t="n">
-        <v>3.080966666666667</v>
+        <v>3.081306666666667</v>
       </c>
       <c r="O524" t="n">
-        <v>88.64541832669322</v>
+        <v>90.43824701195219</v>
       </c>
       <c r="P524" t="n">
-        <v>94.31137724550898</v>
+        <v>95.20958083832335</v>
       </c>
       <c r="Q524" t="n">
         <v>1.4447</v>
       </c>
       <c r="R524" t="n">
-        <v>4.52</v>
+        <v>4.41</v>
       </c>
       <c r="S524" t="n">
-        <v>3.075299999999999</v>
+        <v>2.9653</v>
       </c>
       <c r="T524" t="n">
-        <v>3.075299999999999</v>
+        <v>2.9653</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.308372464934357</v>
+        <v>-4.228679317263247</v>
       </c>
       <c r="V524" t="n">
         <v>6.4705</v>
@@ -85872,10 +85872,10 @@
         <v>-3.105764425058066</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.1708449770707166</v>
+        <v>-0.2774286362031253</v>
       </c>
       <c r="Y524" t="n">
-        <v>10.4</v>
+        <v>7.2</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85898,19 +85898,19 @@
         <v>98.4126984126984</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4946349770706959</v>
+        <v>-0.6012186362031047</v>
       </c>
       <c r="AG524" t="n">
-        <v>6.96560863532838</v>
+        <v>6.960286806749557</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.2877087978344832</v>
+        <v>-0.2823869692556604</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.701717333219215</v>
+        <v>6.689733508675832</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.02381749572531877</v>
+        <v>-0.01183367118193601</v>
       </c>
       <c r="AK524" t="n">
         <v>6.67981241766514</v>
@@ -85928,10 +85928,10 @@
         <v>0.8318271002604343</v>
       </c>
       <c r="AP524" t="n">
-        <v>0.597068793361774</v>
+        <v>0.6974384969722904</v>
       </c>
       <c r="AQ524" t="n">
-        <v>72.66693227091633</v>
+        <v>73.66294820717131</v>
       </c>
       <c r="AR524" t="n">
         <v>-0.004031509296337254</v>
@@ -85958,10 +85958,10 @@
         <v>0.8</v>
       </c>
       <c r="AZ524" t="n">
-        <v>53.10597609561752</v>
+        <v>54.03227091633465</v>
       </c>
       <c r="BA524" t="n">
-        <v>56.03601676567938</v>
+        <v>56.22127572982281</v>
       </c>
     </row>
   </sheetData>
@@ -86188,7 +86188,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.65</t>
+          <t>4.69</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86203,17 +86203,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>3.44</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>90</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>95</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -86223,12 +86223,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.52</t>
+          <t>4.41</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86238,12 +86238,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.17</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86278,17 +86278,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.49</t>
+          <t>-0.60</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.29</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.02</t>
+          <t>-0.01</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86313,7 +86313,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.60</t>
+          <t>0.70</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-26 18:33 EDT
Score: 55/100
USD/CNY: 6.68
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85359,13 +85359,13 @@
         <v>1.4447</v>
       </c>
       <c r="R521" t="n">
-        <v>4.41</v>
+        <v>4.44</v>
       </c>
       <c r="S521" t="n">
-        <v>2.9653</v>
+        <v>2.9953</v>
       </c>
       <c r="T521" t="n">
-        <v>2.9653</v>
+        <v>2.9953</v>
       </c>
       <c r="U521" t="n">
         <v>-4.228679317263247</v>
@@ -85377,7 +85377,7 @@
         <v>-1.187496659483533</v>
       </c>
       <c r="X521" t="n">
-        <v>1.725434737833242</v>
+        <v>1.755078488835382</v>
       </c>
       <c r="Y521" t="n">
         <v>50.40000000000001</v>
@@ -85403,7 +85403,7 @@
         <v>98.4126984126984</v>
       </c>
       <c r="AF521" t="n">
-        <v>1.400434737833245</v>
+        <v>1.430078488835385</v>
       </c>
       <c r="AG521" t="n">
         <v>6.960286806749557</v>
@@ -85476,25 +85476,25 @@
         </is>
       </c>
       <c r="B522" t="n">
-        <v>4.69</v>
+        <v>4.68</v>
       </c>
       <c r="C522" t="n">
         <v>1.2428</v>
       </c>
       <c r="D522" t="n">
-        <v>3.4448</v>
+        <v>3.4372</v>
       </c>
       <c r="E522" t="n">
         <v>6.677899837493896</v>
       </c>
       <c r="F522" t="n">
-        <v>6.666940212249756</v>
+        <v>6.668000221252441</v>
       </c>
       <c r="G522" t="n">
         <v>6.6586</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.01095962524414062</v>
+        <v>-0.009899616241455078</v>
       </c>
       <c r="I522" t="n">
         <v>101.8099975585938</v>
@@ -85503,37 +85503,37 @@
         <v>0</v>
       </c>
       <c r="K522" t="n">
-        <v>3.4448</v>
+        <v>3.4372</v>
       </c>
       <c r="L522" t="n">
-        <v>3.54268</v>
+        <v>3.5423</v>
       </c>
       <c r="M522" t="n">
-        <v>3.293168333333333</v>
+        <v>3.293041666666666</v>
       </c>
       <c r="N522" t="n">
-        <v>3.087745833333333</v>
+        <v>3.0876825</v>
       </c>
       <c r="O522" t="n">
-        <v>90.23904382470118</v>
+        <v>89.64143426294821</v>
       </c>
       <c r="P522" t="n">
-        <v>95.10978043912176</v>
+        <v>94.81037924151697</v>
       </c>
       <c r="Q522" t="n">
         <v>1.4415</v>
       </c>
       <c r="R522" t="n">
-        <v>4.41</v>
+        <v>4.44</v>
       </c>
       <c r="S522" t="n">
-        <v>2.9685</v>
+        <v>2.9985</v>
       </c>
       <c r="T522" t="n">
-        <v>2.9685</v>
+        <v>2.9985</v>
       </c>
       <c r="U522" t="n">
-        <v>-4.045414416388373</v>
+        <v>-4.065294122942751</v>
       </c>
       <c r="V522" t="n">
         <v>6.4689</v>
@@ -85542,10 +85542,10 @@
         <v>-3.129724053667915</v>
       </c>
       <c r="X522" t="n">
-        <v>-0.2992448844346685</v>
+        <v>-0.2701838016507807</v>
       </c>
       <c r="Y522" t="n">
-        <v>6.800000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="Z522" t="inlineStr">
         <is>
@@ -85568,19 +85568,19 @@
         <v>99.2063492063492</v>
       </c>
       <c r="AF522" t="n">
-        <v>-0.6274448844346692</v>
+        <v>-0.5983838016507814</v>
       </c>
       <c r="AG522" t="n">
-        <v>6.94804856023185</v>
+        <v>6.949376107123539</v>
       </c>
       <c r="AH522" t="n">
-        <v>-0.2701487227379538</v>
+        <v>-0.2714762696296429</v>
       </c>
       <c r="AI522" t="n">
-        <v>6.695342242590616</v>
+        <v>6.69755453909513</v>
       </c>
       <c r="AJ522" t="n">
-        <v>-0.01744240509671968</v>
+        <v>-0.01965470160123317</v>
       </c>
       <c r="AK522" t="n">
         <v>6.670848323321455</v>
@@ -85598,10 +85598,10 @@
         <v>0.8335523217311571</v>
       </c>
       <c r="AP522" t="n">
-        <v>0.6488820223959991</v>
+        <v>0.6303629869717073</v>
       </c>
       <c r="AQ522" t="n">
-        <v>73.86533864541832</v>
+        <v>73.66613545816733</v>
       </c>
       <c r="AR522" t="n">
         <v>-0.004307810306897541</v>
@@ -85628,10 +85628,10 @@
         <v>0.7936507936507936</v>
       </c>
       <c r="AZ522" t="n">
-        <v>54.02104471004869</v>
+        <v>53.75212040725985</v>
       </c>
       <c r="BA522" t="n">
-        <v>55.34352187837826</v>
+        <v>55.28973701782049</v>
       </c>
     </row>
   </sheetData>
@@ -85858,7 +85858,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.69</t>
+          <t>4.68</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -85893,12 +85893,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.41</t>
+          <t>4.44</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -85908,7 +85908,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -85948,7 +85948,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.63</t>
+          <t>-0.60</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -85983,7 +85983,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.65</t>
+          <t>0.63</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-26 19:05 EDT
Score: 55/100
USD/CNY: 6.68
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85488,13 +85488,13 @@
         <v>6.677899837493896</v>
       </c>
       <c r="F522" t="n">
-        <v>6.668000221252441</v>
+        <v>6.666910171508789</v>
       </c>
       <c r="G522" t="n">
         <v>6.6586</v>
       </c>
       <c r="H522" t="n">
-        <v>-0.009899616241455078</v>
+        <v>-0.01098966598510742</v>
       </c>
       <c r="I522" t="n">
         <v>101.8099975585938</v>

</xml_diff>

<commit_message>
auto: data update 2026-10-27 15:46 EDT
Score: 74/100
USD/CNY: 6.68
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85653,13 +85653,13 @@
         <v>6.677899837493896</v>
       </c>
       <c r="F523" t="n">
-        <v>6.6642</v>
+        <v>6.664</v>
       </c>
       <c r="G523" t="n">
         <v>6.6549</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.01369983749389636</v>
+        <v>-0.01389983749389678</v>
       </c>
       <c r="I523" t="n">
         <v>101.9599990844727</v>

</xml_diff>

<commit_message>
auto: data update 2026-10-27 18:54 EDT
Score: 54/100
USD/CNY: 6.68
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85653,13 +85653,13 @@
         <v>6.677899837493896</v>
       </c>
       <c r="F523" t="n">
-        <v>6.664539813995361</v>
+        <v>6.664529800415039</v>
       </c>
       <c r="G523" t="n">
         <v>6.6549</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.01336002349853516</v>
+        <v>-0.01337003707885742</v>
       </c>
       <c r="I523" t="n">
         <v>101.9599990844727</v>

</xml_diff>

<commit_message>
auto: data update 2026-10-28 15:11 EDT
Score: 53/100
USD/CNY: 6.67
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA523"/>
+  <dimension ref="A1:BA524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85650,22 +85650,22 @@
         <v>3.4597</v>
       </c>
       <c r="E523" t="n">
-        <v>6.677899837493896</v>
+        <v>6.670000076293945</v>
       </c>
       <c r="F523" t="n">
-        <v>6.664529800415039</v>
+        <v>6.7778000831604</v>
       </c>
       <c r="G523" t="n">
         <v>6.6549</v>
       </c>
       <c r="H523" t="n">
-        <v>-0.01337003707885742</v>
+        <v>0.1078000068664551</v>
       </c>
       <c r="I523" t="n">
-        <v>101.9599990844727</v>
+        <v>102.3199996948242</v>
       </c>
       <c r="J523" t="n">
-        <v>0</v>
+        <v>0.003530802408631795</v>
       </c>
       <c r="K523" t="n">
         <v>3.4597</v>
@@ -85698,19 +85698,19 @@
         <v>3.029</v>
       </c>
       <c r="U523" t="n">
-        <v>-3.873278136689549</v>
+        <v>-3.996302736831967</v>
       </c>
       <c r="V523" t="n">
-        <v>6.4683</v>
+        <v>6.5986</v>
       </c>
       <c r="W523" t="n">
-        <v>-3.138708914396593</v>
+        <v>-1.070465899209061</v>
       </c>
       <c r="X523" t="n">
-        <v>-0.2500092028701273</v>
+        <v>1.910684275096286</v>
       </c>
       <c r="Y523" t="n">
-        <v>8</v>
+        <v>51.6</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85718,40 +85718,40 @@
         </is>
       </c>
       <c r="AA523" t="n">
-        <v>1.75</v>
+        <v>1.76576</v>
       </c>
       <c r="AB523" t="n">
-        <v>1.63606</v>
+        <v>1.60727</v>
       </c>
       <c r="AC523" t="n">
-        <v>1.37879</v>
+        <v>1.37788</v>
       </c>
       <c r="AD523" t="n">
-        <v>0.3089999999999999</v>
+        <v>0.3247599999999999</v>
       </c>
       <c r="AE523" t="n">
-        <v>94.84126984126983</v>
+        <v>98.01587301587301</v>
       </c>
       <c r="AF523" t="n">
-        <v>-0.559009202870131</v>
+        <v>1.585924275096295</v>
       </c>
       <c r="AG523" t="n">
         <v>6.936553471889574</v>
       </c>
       <c r="AH523" t="n">
-        <v>-0.258653634395678</v>
+        <v>-0.2665533955956292</v>
       </c>
       <c r="AI523" t="n">
-        <v>6.694928764155931</v>
+        <v>6.705818145853503</v>
       </c>
       <c r="AJ523" t="n">
-        <v>-0.01702892666203404</v>
+        <v>-0.03581806955955802</v>
       </c>
       <c r="AK523" t="n">
         <v>6.673122869741766</v>
       </c>
       <c r="AL523" t="n">
-        <v>0.004776967752130545</v>
+        <v>-0.003122793447820627</v>
       </c>
       <c r="AM523" t="n">
         <v>-0.2887745258469642</v>
@@ -85763,40 +85763,205 @@
         <v>0.8349576802847257</v>
       </c>
       <c r="AP523" t="n">
-        <v>0.6508450706654625</v>
+        <v>0.4935685055213775</v>
       </c>
       <c r="AQ523" t="n">
-        <v>75.26533864541832</v>
+        <v>72.27330677290837</v>
       </c>
       <c r="AR523" t="n">
-        <v>-0.004600800498822249</v>
+        <v>-0.005817121415643785</v>
       </c>
       <c r="AS523" t="n">
-        <v>6.7778000831604</v>
+        <v>6.777660873203974</v>
       </c>
       <c r="AT523" t="n">
-        <v>-0.1229000831603999</v>
+        <v>-0.1227608732039736</v>
       </c>
       <c r="AU523" t="n">
         <v>-0.1229000831603999</v>
       </c>
       <c r="AV523" t="n">
-        <v>-0.09804149159373013</v>
+        <v>-0.0980345310959088</v>
       </c>
       <c r="AW523" t="n">
-        <v>-0.07783900085319037</v>
+        <v>-0.07783668068724993</v>
       </c>
       <c r="AX523" t="n">
-        <v>0.08587408670742677</v>
+        <v>0.0858737386825357</v>
       </c>
       <c r="AY523" t="n">
         <v>0.7874015748031495</v>
       </c>
       <c r="AZ523" t="n">
-        <v>54.50857859898986</v>
+        <v>53.61096903723688</v>
       </c>
       <c r="BA523" t="n">
-        <v>54.33101592748196</v>
+        <v>54.15149401513137</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B524" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C524" t="n">
+        <v>1.233</v>
+      </c>
+      <c r="D524" t="n">
+        <v>3.4597</v>
+      </c>
+      <c r="E524" t="n">
+        <v>6.670000076293945</v>
+      </c>
+      <c r="F524" t="n">
+        <v>6.661849975585938</v>
+      </c>
+      <c r="G524" t="n">
+        <v>6.6546</v>
+      </c>
+      <c r="H524" t="n">
+        <v>-0.008150100708007812</v>
+      </c>
+      <c r="I524" t="n">
+        <v>102.3199996948242</v>
+      </c>
+      <c r="J524" t="n">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>3.4597</v>
+      </c>
+      <c r="L524" t="n">
+        <v>3.526045</v>
+      </c>
+      <c r="M524" t="n">
+        <v>3.310638333333333</v>
+      </c>
+      <c r="N524" t="n">
+        <v>3.100088333333333</v>
+      </c>
+      <c r="O524" t="n">
+        <v>90.23904382470118</v>
+      </c>
+      <c r="P524" t="n">
+        <v>95.10978043912176</v>
+      </c>
+      <c r="Q524" t="n">
+        <v>1.438</v>
+      </c>
+      <c r="R524" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="S524" t="n">
+        <v>3.032</v>
+      </c>
+      <c r="T524" t="n">
+        <v>3.032</v>
+      </c>
+      <c r="U524" t="n">
+        <v>-4.044641668334491</v>
+      </c>
+      <c r="V524" t="n">
+        <v>6.4665</v>
+      </c>
+      <c r="W524" t="n">
+        <v>-3.050975621682694</v>
+      </c>
+      <c r="X524" t="n">
+        <v>-0.155354231971927</v>
+      </c>
+      <c r="Y524" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="Z524" t="inlineStr">
+        <is>
+          <t>market_1y</t>
+        </is>
+      </c>
+      <c r="AA524" t="n">
+        <v>1.76576</v>
+      </c>
+      <c r="AB524" t="n">
+        <v>1.60727</v>
+      </c>
+      <c r="AC524" t="n">
+        <v>1.37788</v>
+      </c>
+      <c r="AD524" t="n">
+        <v>0.3277600000000001</v>
+      </c>
+      <c r="AE524" t="n">
+        <v>99.2063492063492</v>
+      </c>
+      <c r="AF524" t="n">
+        <v>-0.4831142319719151</v>
+      </c>
+      <c r="AG524" t="n">
+        <v>6.939777678657673</v>
+      </c>
+      <c r="AH524" t="n">
+        <v>-0.2697776023637273</v>
+      </c>
+      <c r="AI524" t="n">
+        <v>6.704611868127235</v>
+      </c>
+      <c r="AJ524" t="n">
+        <v>-0.03461179183328955</v>
+      </c>
+      <c r="AK524" t="n">
+        <v>6.668492963897435</v>
+      </c>
+      <c r="AL524" t="n">
+        <v>0.001507112396510024</v>
+      </c>
+      <c r="AM524" t="n">
+        <v>-0.2865822231249923</v>
+      </c>
+      <c r="AN524" t="n">
+        <v>0.02940685489086397</v>
+      </c>
+      <c r="AO524" t="n">
+        <v>0.8360274389571491</v>
+      </c>
+      <c r="AP524" t="n">
+        <v>0.5026988995922758</v>
+      </c>
+      <c r="AQ524" t="n">
+        <v>72.07330677290837</v>
+      </c>
+      <c r="AR524" t="n">
+        <v>-0.005837384719744309</v>
+      </c>
+      <c r="AS524" t="n">
+        <v>6.7778000831604</v>
+      </c>
+      <c r="AT524" t="n">
+        <v>-0.1232000831604001</v>
+      </c>
+      <c r="AU524" t="n">
+        <v>-0.1232000831604001</v>
+      </c>
+      <c r="AV524" t="n">
+        <v>-0.1001930972634826</v>
+      </c>
+      <c r="AW524" t="n">
+        <v>-0.0792095169386479</v>
+      </c>
+      <c r="AX524" t="n">
+        <v>0.08686726937274343</v>
+      </c>
+      <c r="AY524" t="n">
+        <v>0.78125</v>
+      </c>
+      <c r="AZ524" t="n">
+        <v>53.47909487051793</v>
+      </c>
+      <c r="BA524" t="n">
+        <v>53.20272114522886</v>
       </c>
     </row>
   </sheetData>
@@ -86003,12 +86168,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6.68</t>
+          <t>6.67</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -86028,12 +86193,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>101.96</t>
+          <t>102.32</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -86073,12 +86238,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.16</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86088,12 +86253,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1.64</t>
+          <t>1.61</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -86103,27 +86268,27 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>0.31</t>
+          <t>0.33</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>99</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.56</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.02</t>
+          <t>-0.03</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86133,27 +86298,27 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>-0.289</t>
+          <t>-0.287</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0.0302</t>
+          <t>0.0294</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.835</t>
+          <t>0.836</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.65</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>-0.005</t>
+          <t>-0.006</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -86183,7 +86348,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: data update 2026-10-29 18:40 EDT
Score: 53/100
USD/CNY: 6.67
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85689,13 +85689,13 @@
         <v>1.438</v>
       </c>
       <c r="R523" t="n">
-        <v>4.5</v>
+        <v>4.47</v>
       </c>
       <c r="S523" t="n">
-        <v>3.062</v>
+        <v>3.032</v>
       </c>
       <c r="T523" t="n">
-        <v>3.062</v>
+        <v>3.032</v>
       </c>
       <c r="U523" t="n">
         <v>-4.135514519473479</v>
@@ -85707,7 +85707,7 @@
         <v>-1.040795125219807</v>
       </c>
       <c r="X523" t="n">
-        <v>1.974369094145279</v>
+        <v>1.944681332682863</v>
       </c>
       <c r="Y523" t="n">
         <v>52</v>
@@ -85733,7 +85733,7 @@
         <v>99.2063492063492</v>
       </c>
       <c r="AF523" t="n">
-        <v>1.644789094145294</v>
+        <v>1.615101332682878</v>
       </c>
       <c r="AG523" t="n">
         <v>6.94375633856086</v>
@@ -85806,25 +85806,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.67</v>
+        <v>4.61</v>
       </c>
       <c r="C524" t="n">
         <v>1.2218</v>
       </c>
       <c r="D524" t="n">
-        <v>3.437</v>
+        <v>3.3882</v>
       </c>
       <c r="E524" t="n">
         <v>6.668000221252441</v>
       </c>
       <c r="F524" t="n">
-        <v>6.656539916992188</v>
+        <v>6.656239986419678</v>
       </c>
       <c r="G524" t="n">
         <v>6.650399999999999</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01146030426025391</v>
+        <v>-0.01176023483276367</v>
       </c>
       <c r="I524" t="n">
         <v>102.1900024414062</v>
@@ -85833,37 +85833,37 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>3.437</v>
+        <v>3.3882</v>
       </c>
       <c r="L524" t="n">
-        <v>3.516084999999999</v>
+        <v>3.513644999999999</v>
       </c>
       <c r="M524" t="n">
-        <v>3.317623333333333</v>
+        <v>3.31681</v>
       </c>
       <c r="N524" t="n">
-        <v>3.105826666666667</v>
+        <v>3.105420000000001</v>
       </c>
       <c r="O524" t="n">
-        <v>88.64541832669322</v>
+        <v>86.85258964143426</v>
       </c>
       <c r="P524" t="n">
-        <v>94.31137724550898</v>
+        <v>93.41317365269461</v>
       </c>
       <c r="Q524" t="n">
         <v>1.4378</v>
       </c>
       <c r="R524" t="n">
-        <v>4.5</v>
+        <v>4.47</v>
       </c>
       <c r="S524" t="n">
-        <v>3.0622</v>
+        <v>3.0322</v>
       </c>
       <c r="T524" t="n">
-        <v>3.0622</v>
+        <v>3.0322</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.121068874289444</v>
+        <v>-4.240542265352092</v>
       </c>
       <c r="V524" t="n">
         <v>6.4648</v>
@@ -85872,10 +85872,10 @@
         <v>-3.047393738902338</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.1223264571529548</v>
+        <v>-0.1514122390312789</v>
       </c>
       <c r="Y524" t="n">
-        <v>12.8</v>
+        <v>11.2</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85898,19 +85898,19 @@
         <v>99.2063492063492</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4521064571529454</v>
+        <v>-0.4811922390312695</v>
       </c>
       <c r="AG524" t="n">
-        <v>6.942793102908027</v>
+        <v>6.950759588888422</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.2747928816555856</v>
+        <v>-0.2827593676359808</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.706064312285513</v>
+        <v>6.719936548684691</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.03806409103307118</v>
+        <v>-0.05193632743224974</v>
       </c>
       <c r="AK524" t="n">
         <v>6.67398568839331</v>
@@ -85928,10 +85928,10 @@
         <v>0.8376262141503689</v>
       </c>
       <c r="AP524" t="n">
-        <v>0.4730761749050949</v>
+        <v>0.356912530196431</v>
       </c>
       <c r="AQ524" t="n">
-        <v>71.47490039840638</v>
+        <v>70.27649402390438</v>
       </c>
       <c r="AR524" t="n">
         <v>-0.005576696558794205</v>
@@ -85958,10 +85958,10 @@
         <v>0.7751937984496124</v>
       </c>
       <c r="AZ524" t="n">
-        <v>52.73968436332191</v>
+        <v>51.75267241113067</v>
       </c>
       <c r="BA524" t="n">
-        <v>53.31755301853584</v>
+        <v>53.12015062809759</v>
       </c>
     </row>
   </sheetData>
@@ -86188,7 +86188,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.67</t>
+          <t>4.61</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86203,17 +86203,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.44</t>
+          <t>3.39</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>87</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>93</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -86223,12 +86223,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>4.47</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.06</t>
+          <t>3.03</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86238,12 +86238,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.12</t>
+          <t>-0.15</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86278,17 +86278,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.45</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>-0.27</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.04</t>
+          <t>-0.05</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86313,7 +86313,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.36</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">

</xml_diff>

<commit_message>
auto: data update 2026-10-30 18:10 EDT
Score: 52/100
USD/CNY: 6.67
</commit_message>
<xml_diff>
--- a/docs/usdcny_tracker.xlsx
+++ b/docs/usdcny_tracker.xlsx
@@ -85689,13 +85689,13 @@
         <v>1.4378</v>
       </c>
       <c r="R523" t="n">
-        <v>4.47</v>
+        <v>4.42</v>
       </c>
       <c r="S523" t="n">
-        <v>3.0322</v>
+        <v>2.9822</v>
       </c>
       <c r="T523" t="n">
-        <v>3.0322</v>
+        <v>2.9822</v>
       </c>
       <c r="U523" t="n">
         <v>-4.271822745880572</v>
@@ -85707,10 +85707,10 @@
         <v>-1.011099467331533</v>
       </c>
       <c r="X523" t="n">
-        <v>1.975904386478744</v>
+        <v>1.926409936212425</v>
       </c>
       <c r="Y523" t="n">
-        <v>52.40000000000001</v>
+        <v>51.6</v>
       </c>
       <c r="Z523" t="inlineStr">
         <is>
@@ -85733,7 +85733,7 @@
         <v>100</v>
       </c>
       <c r="AF523" t="n">
-        <v>1.643404386478742</v>
+        <v>1.593909936212423</v>
       </c>
       <c r="AG523" t="n">
         <v>6.950759588888422</v>
@@ -85806,25 +85806,25 @@
         </is>
       </c>
       <c r="B524" t="n">
-        <v>4.61</v>
+        <v>4.56</v>
       </c>
       <c r="C524" t="n">
         <v>1.2457</v>
       </c>
       <c r="D524" t="n">
-        <v>3.3882</v>
+        <v>3.314299999999999</v>
       </c>
       <c r="E524" t="n">
         <v>6.665999889373779</v>
       </c>
       <c r="F524" t="n">
-        <v>6.653689861297607</v>
+        <v>6.651529788970947</v>
       </c>
       <c r="G524" t="n">
         <v>6.6435</v>
       </c>
       <c r="H524" t="n">
-        <v>-0.01231002807617188</v>
+        <v>-0.01447010040283203</v>
       </c>
       <c r="I524" t="n">
         <v>102.0400009155273</v>
@@ -85833,37 +85833,37 @@
         <v>0</v>
       </c>
       <c r="K524" t="n">
-        <v>3.3882</v>
+        <v>3.314299999999999</v>
       </c>
       <c r="L524" t="n">
-        <v>3.50238</v>
+        <v>3.498685</v>
       </c>
       <c r="M524" t="n">
-        <v>3.324318333333333</v>
+        <v>3.323086666666667</v>
       </c>
       <c r="N524" t="n">
-        <v>3.1101825</v>
+        <v>3.109566666666667</v>
       </c>
       <c r="O524" t="n">
-        <v>86.65338645418326</v>
+        <v>85.65737051792829</v>
       </c>
       <c r="P524" t="n">
-        <v>93.31337325349301</v>
+        <v>92.81437125748504</v>
       </c>
       <c r="Q524" t="n">
         <v>1.438</v>
       </c>
       <c r="R524" t="n">
-        <v>4.47</v>
+        <v>4.42</v>
       </c>
       <c r="S524" t="n">
-        <v>3.032</v>
+        <v>2.982</v>
       </c>
       <c r="T524" t="n">
-        <v>3.032</v>
+        <v>2.982</v>
       </c>
       <c r="U524" t="n">
-        <v>-4.283048382340017</v>
+        <v>-4.382807355335427</v>
       </c>
       <c r="V524" t="n">
         <v>6.4619</v>
@@ -85872,10 +85872,10 @@
         <v>-3.061804571871252</v>
       </c>
       <c r="X524" t="n">
-        <v>-0.1666672362339083</v>
+        <v>-0.2151363339479628</v>
       </c>
       <c r="Y524" t="n">
-        <v>10.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Z524" t="inlineStr">
         <is>
@@ -85898,19 +85898,19 @@
         <v>99.60317460317459</v>
       </c>
       <c r="AF524" t="n">
-        <v>-0.4989672362339048</v>
+        <v>-0.5474363339479593</v>
       </c>
       <c r="AG524" t="n">
-        <v>6.95150788980239</v>
+        <v>6.958157822831905</v>
       </c>
       <c r="AH524" t="n">
-        <v>-0.285508000428611</v>
+        <v>-0.2921579334581255</v>
       </c>
       <c r="AI524" t="n">
-        <v>6.714384287003274</v>
+        <v>6.735221785383466</v>
       </c>
       <c r="AJ524" t="n">
-        <v>-0.04838439762949509</v>
+        <v>-0.06922189600968665</v>
       </c>
       <c r="AK524" t="n">
         <v>6.685125514440118</v>
@@ -85928,10 +85928,10 @@
         <v>0.8394257868452498</v>
       </c>
       <c r="AP524" t="n">
-        <v>0.3864252069506037</v>
+        <v>0.2118629975881758</v>
       </c>
       <c r="AQ524" t="n">
-        <v>70.27649402390438</v>
+        <v>68.28366533864542</v>
       </c>
       <c r="AR524" t="n">
         <v>-0.005555486782516207</v>
@@ -85958,10 +85958,10 @@
         <v>0.7692307692307693</v>
       </c>
       <c r="AZ524" t="n">
-        <v>51.68086423536622</v>
+        <v>50.73441005209929</v>
       </c>
       <c r="BA524" t="n">
-        <v>52.68572586560907</v>
+        <v>52.49643502895569</v>
       </c>
     </row>
   </sheetData>
@@ -86188,7 +86188,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4.61</t>
+          <t>4.56</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -86203,12 +86203,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.39</t>
+          <t>3.31</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>86</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -86223,12 +86223,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4.47</t>
+          <t>4.42</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.03</t>
+          <t>2.98</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -86238,12 +86238,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>-0.17</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -86278,7 +86278,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>-0.50</t>
+          <t>-0.55</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -86288,7 +86288,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>-0.05</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -86313,7 +86313,7 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>0.39</t>
+          <t>0.21</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -86348,7 +86348,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>52</t>
         </is>
       </c>
     </row>

</xml_diff>